<commit_message>
updated farsi + translated Reference phrase
</commit_message>
<xml_diff>
--- a/assets/LadenburgConsensuStatements.xlsx
+++ b/assets/LadenburgConsensuStatements.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/mspitschan/Projects/LadenburgConsensusStatements/assets/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/zauner/Documents/Arbeit/12-TUM/Repos_Misc/2024-04_Ladenburg_Roundtable/LCS/assets/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2D1A86B6-749A-A242-A218-22E042E258AA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6E1478FA-EF4D-9F43-88B0-F0DA08DA0C80}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="920" yWindow="880" windowWidth="17540" windowHeight="22500" firstSheet="7" activeTab="14" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="11880" yWindow="2680" windowWidth="25380" windowHeight="21660" activeTab="12" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="English" sheetId="4" r:id="rId1"/>
@@ -50,7 +50,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1931" uniqueCount="1484">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1907" uniqueCount="1481">
   <si>
     <t>Number</t>
   </si>
@@ -7254,46 +7254,37 @@
     <t>Artemide</t>
   </si>
   <si>
-    <t>Leiden University Medical Center</t>
-  </si>
-  <si>
-    <t>Chrono@Work &amp; University of Groningen</t>
-  </si>
-  <si>
-    <t>National Research Council of Canada</t>
-  </si>
-  <si>
-    <t>Stanford University</t>
-  </si>
-  <si>
-    <t>Renske</t>
-  </si>
-  <si>
-    <t>Lok</t>
-  </si>
-  <si>
-    <t>Gordijn</t>
-  </si>
-  <si>
-    <t>Jennifer A.</t>
-  </si>
-  <si>
-    <t>Veitch</t>
-  </si>
-  <si>
-    <t>rlok@stanford.edu</t>
-  </si>
-  <si>
-    <t>Jennifer.Veitch@nrc-cnrc.gc.ca</t>
-  </si>
-  <si>
-    <t>L.Kervezee@lumc.nl</t>
-  </si>
-  <si>
-    <t>0000-0003-3183-4537</t>
-  </si>
-  <si>
-    <t>0000-0003-1684-5625</t>
+    <t>Kaynaklar</t>
+  </si>
+  <si>
+    <t>Referências</t>
+  </si>
+  <si>
+    <t>Bibliografia</t>
+  </si>
+  <si>
+    <t>참고문헌</t>
+  </si>
+  <si>
+    <t>Riferimenti</t>
+  </si>
+  <si>
+    <t>Références</t>
+  </si>
+  <si>
+    <t>参考文献 </t>
+  </si>
+  <si>
+    <t>Referenties</t>
+  </si>
+  <si>
+    <t>منابع</t>
+  </si>
+  <si>
+    <t>Referencer</t>
+  </si>
+  <si>
+    <t>Seznam literatury</t>
   </si>
 </sst>
 </file>
@@ -8447,7 +8438,7 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="44">
+  <cellStyleXfs count="45">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="1" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0"/>
@@ -8494,8 +8485,9 @@
     <xf numFmtId="0" fontId="42" fillId="0" borderId="0">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="25" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="137">
+  <cellXfs count="138">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
@@ -8831,6 +8823,7 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="72" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="25" fillId="0" borderId="0" xfId="44"/>
     <xf numFmtId="0" fontId="31" fillId="33" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -8846,51 +8839,52 @@
       <alignment horizontal="center"/>
     </xf>
   </cellXfs>
-  <cellStyles count="44">
-    <cellStyle name="20% - Accent1" xfId="19" builtinId="30" customBuiltin="1"/>
-    <cellStyle name="20% - Accent2" xfId="23" builtinId="34" customBuiltin="1"/>
-    <cellStyle name="20% - Accent3" xfId="27" builtinId="38" customBuiltin="1"/>
-    <cellStyle name="20% - Accent4" xfId="31" builtinId="42" customBuiltin="1"/>
-    <cellStyle name="20% - Accent5" xfId="35" builtinId="46" customBuiltin="1"/>
-    <cellStyle name="20% - Accent6" xfId="39" builtinId="50" customBuiltin="1"/>
-    <cellStyle name="40% - Accent1" xfId="20" builtinId="31" customBuiltin="1"/>
-    <cellStyle name="40% - Accent2" xfId="24" builtinId="35" customBuiltin="1"/>
-    <cellStyle name="40% - Accent3" xfId="28" builtinId="39" customBuiltin="1"/>
-    <cellStyle name="40% - Accent4" xfId="32" builtinId="43" customBuiltin="1"/>
-    <cellStyle name="40% - Accent5" xfId="36" builtinId="47" customBuiltin="1"/>
-    <cellStyle name="40% - Accent6" xfId="40" builtinId="51" customBuiltin="1"/>
-    <cellStyle name="60% - Accent1" xfId="21" builtinId="32" customBuiltin="1"/>
-    <cellStyle name="60% - Accent2" xfId="25" builtinId="36" customBuiltin="1"/>
-    <cellStyle name="60% - Accent3" xfId="29" builtinId="40" customBuiltin="1"/>
-    <cellStyle name="60% - Accent4" xfId="33" builtinId="44" customBuiltin="1"/>
-    <cellStyle name="60% - Accent5" xfId="37" builtinId="48" customBuiltin="1"/>
-    <cellStyle name="60% - Accent6" xfId="41" builtinId="52" customBuiltin="1"/>
-    <cellStyle name="Accent1" xfId="18" builtinId="29" customBuiltin="1"/>
-    <cellStyle name="Accent2" xfId="22" builtinId="33" customBuiltin="1"/>
-    <cellStyle name="Accent3" xfId="26" builtinId="37" customBuiltin="1"/>
-    <cellStyle name="Accent4" xfId="30" builtinId="41" customBuiltin="1"/>
-    <cellStyle name="Accent5" xfId="34" builtinId="45" customBuiltin="1"/>
-    <cellStyle name="Accent6" xfId="38" builtinId="49" customBuiltin="1"/>
-    <cellStyle name="Bad" xfId="7" builtinId="27" customBuiltin="1"/>
-    <cellStyle name="Calculation" xfId="11" builtinId="22" customBuiltin="1"/>
-    <cellStyle name="Check Cell" xfId="13" builtinId="23" customBuiltin="1"/>
-    <cellStyle name="Explanatory Text" xfId="16" builtinId="53" customBuiltin="1"/>
-    <cellStyle name="Good" xfId="6" builtinId="26" customBuiltin="1"/>
-    <cellStyle name="Heading 1" xfId="2" builtinId="16" customBuiltin="1"/>
-    <cellStyle name="Heading 2" xfId="3" builtinId="17" customBuiltin="1"/>
-    <cellStyle name="Heading 3" xfId="4" builtinId="18" customBuiltin="1"/>
-    <cellStyle name="Heading 4" xfId="5" builtinId="19" customBuiltin="1"/>
-    <cellStyle name="Hyperlink" xfId="42" xr:uid="{B2D74732-8E41-314C-B68A-0975ED16242F}"/>
-    <cellStyle name="Input" xfId="9" builtinId="20" customBuiltin="1"/>
-    <cellStyle name="Linked Cell" xfId="12" builtinId="24" customBuiltin="1"/>
+  <cellStyles count="45">
+    <cellStyle name="20 % - Akzent1" xfId="19" builtinId="30" customBuiltin="1"/>
+    <cellStyle name="20 % - Akzent2" xfId="23" builtinId="34" customBuiltin="1"/>
+    <cellStyle name="20 % - Akzent3" xfId="27" builtinId="38" customBuiltin="1"/>
+    <cellStyle name="20 % - Akzent4" xfId="31" builtinId="42" customBuiltin="1"/>
+    <cellStyle name="20 % - Akzent5" xfId="35" builtinId="46" customBuiltin="1"/>
+    <cellStyle name="20 % - Akzent6" xfId="39" builtinId="50" customBuiltin="1"/>
+    <cellStyle name="40 % - Akzent1" xfId="20" builtinId="31" customBuiltin="1"/>
+    <cellStyle name="40 % - Akzent2" xfId="24" builtinId="35" customBuiltin="1"/>
+    <cellStyle name="40 % - Akzent3" xfId="28" builtinId="39" customBuiltin="1"/>
+    <cellStyle name="40 % - Akzent4" xfId="32" builtinId="43" customBuiltin="1"/>
+    <cellStyle name="40 % - Akzent5" xfId="36" builtinId="47" customBuiltin="1"/>
+    <cellStyle name="40 % - Akzent6" xfId="40" builtinId="51" customBuiltin="1"/>
+    <cellStyle name="60 % - Akzent1" xfId="21" builtinId="32" customBuiltin="1"/>
+    <cellStyle name="60 % - Akzent2" xfId="25" builtinId="36" customBuiltin="1"/>
+    <cellStyle name="60 % - Akzent3" xfId="29" builtinId="40" customBuiltin="1"/>
+    <cellStyle name="60 % - Akzent4" xfId="33" builtinId="44" customBuiltin="1"/>
+    <cellStyle name="60 % - Akzent5" xfId="37" builtinId="48" customBuiltin="1"/>
+    <cellStyle name="60 % - Akzent6" xfId="41" builtinId="52" customBuiltin="1"/>
+    <cellStyle name="Akzent1" xfId="18" builtinId="29" customBuiltin="1"/>
+    <cellStyle name="Akzent2" xfId="22" builtinId="33" customBuiltin="1"/>
+    <cellStyle name="Akzent3" xfId="26" builtinId="37" customBuiltin="1"/>
+    <cellStyle name="Akzent4" xfId="30" builtinId="41" customBuiltin="1"/>
+    <cellStyle name="Akzent5" xfId="34" builtinId="45" customBuiltin="1"/>
+    <cellStyle name="Akzent6" xfId="38" builtinId="49" customBuiltin="1"/>
+    <cellStyle name="Ausgabe" xfId="10" builtinId="21" customBuiltin="1"/>
+    <cellStyle name="Berechnung" xfId="11" builtinId="22" customBuiltin="1"/>
+    <cellStyle name="Eingabe" xfId="9" builtinId="20" customBuiltin="1"/>
+    <cellStyle name="Ergebnis" xfId="17" builtinId="25" customBuiltin="1"/>
+    <cellStyle name="Erklärender Text" xfId="16" builtinId="53" customBuiltin="1"/>
+    <cellStyle name="Gut" xfId="6" builtinId="26" customBuiltin="1"/>
+    <cellStyle name="Hyperlink" xfId="44" xr:uid="{B2D74732-8E41-314C-B68A-0975ED16242F}"/>
+    <cellStyle name="Link" xfId="42" builtinId="8"/>
     <cellStyle name="Neutral" xfId="8" builtinId="28" customBuiltin="1"/>
-    <cellStyle name="Normal" xfId="0" builtinId="0"/>
-    <cellStyle name="Note" xfId="15" builtinId="10" customBuiltin="1"/>
-    <cellStyle name="Output" xfId="10" builtinId="21" customBuiltin="1"/>
+    <cellStyle name="Notiz" xfId="15" builtinId="10" customBuiltin="1"/>
+    <cellStyle name="Schlecht" xfId="7" builtinId="27" customBuiltin="1"/>
+    <cellStyle name="Standard" xfId="0" builtinId="0"/>
     <cellStyle name="Standard 2" xfId="43" xr:uid="{70AE8D79-DF60-5941-BC6B-2804C19A889C}"/>
-    <cellStyle name="Title" xfId="1" builtinId="15" customBuiltin="1"/>
-    <cellStyle name="Total" xfId="17" builtinId="25" customBuiltin="1"/>
-    <cellStyle name="Warning Text" xfId="14" builtinId="11" customBuiltin="1"/>
+    <cellStyle name="Überschrift" xfId="1" builtinId="15" customBuiltin="1"/>
+    <cellStyle name="Überschrift 1" xfId="2" builtinId="16" customBuiltin="1"/>
+    <cellStyle name="Überschrift 2" xfId="3" builtinId="17" customBuiltin="1"/>
+    <cellStyle name="Überschrift 3" xfId="4" builtinId="18" customBuiltin="1"/>
+    <cellStyle name="Überschrift 4" xfId="5" builtinId="19" customBuiltin="1"/>
+    <cellStyle name="Verknüpfte Zelle" xfId="12" builtinId="24" customBuiltin="1"/>
+    <cellStyle name="Warnender Text" xfId="14" builtinId="11" customBuiltin="1"/>
+    <cellStyle name="Zelle überprüfen" xfId="13" builtinId="23" customBuiltin="1"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
@@ -8906,9 +8900,9 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office 2013 - 2022 Theme">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office 2013 – 2022-Design">
   <a:themeElements>
-    <a:clrScheme name="Office 2013 - 2022">
+    <a:clrScheme name="Office 2013 – 2022">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -8946,7 +8940,7 @@
         <a:srgbClr val="954F72"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office 2013 - 2022">
+    <a:fontScheme name="Office 2013 – 2022">
       <a:majorFont>
         <a:latin typeface="Calibri Light" panose="020F0302020204030204"/>
         <a:ea typeface=""/>
@@ -9052,7 +9046,7 @@
         <a:font script="Tfng" typeface="Ebrima"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office 2013 - 2022">
+    <a:fmtScheme name="Office 2013 – 2022">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -9711,7 +9705,7 @@
         <v>193</v>
       </c>
     </row>
-    <row r="26" spans="1:6" ht="119">
+    <row r="26" spans="1:6" ht="136">
       <c r="A26" t="s">
         <v>206</v>
       </c>
@@ -9758,7 +9752,7 @@
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E7A6E799-3425-7049-AD78-3DEC34B23389}">
-  <dimension ref="A1:E27"/>
+  <dimension ref="A1:F27"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="10.6640625" defaultRowHeight="15.75" customHeight="1"/>
   <cols>
     <col min="1" max="1" width="24.33203125" style="24" customWidth="1"/>
@@ -9766,7 +9760,7 @@
     <col min="3" max="5" width="42.33203125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" ht="16">
+    <row r="1" spans="1:6" ht="16">
       <c r="A1" t="s">
         <v>1051</v>
       </c>
@@ -9782,8 +9776,11 @@
       <c r="E1" t="s">
         <v>1054</v>
       </c>
-    </row>
-    <row r="2" spans="1:5" ht="93" customHeight="1">
+      <c r="F1" s="108" t="s">
+        <v>1477</v>
+      </c>
+    </row>
+    <row r="2" spans="1:6" ht="93" customHeight="1">
       <c r="A2" s="116" t="s">
         <v>202</v>
       </c>
@@ -9800,7 +9797,7 @@
         <v>1175</v>
       </c>
     </row>
-    <row r="3" spans="1:5" ht="85">
+    <row r="3" spans="1:6" ht="85">
       <c r="A3" s="116" t="s">
         <v>202</v>
       </c>
@@ -9817,7 +9814,7 @@
         <v>1172</v>
       </c>
     </row>
-    <row r="4" spans="1:5" ht="136">
+    <row r="4" spans="1:6" ht="153">
       <c r="A4" s="116" t="s">
         <v>202</v>
       </c>
@@ -9834,7 +9831,7 @@
         <v>1169</v>
       </c>
     </row>
-    <row r="5" spans="1:5" ht="117.75" customHeight="1">
+    <row r="5" spans="1:6" ht="117.75" customHeight="1">
       <c r="A5" s="116" t="s">
         <v>202</v>
       </c>
@@ -9851,7 +9848,7 @@
         <v>1166</v>
       </c>
     </row>
-    <row r="6" spans="1:5" ht="150" customHeight="1">
+    <row r="6" spans="1:6" ht="150" customHeight="1">
       <c r="A6" s="116" t="s">
         <v>202</v>
       </c>
@@ -9868,7 +9865,7 @@
         <v>1163</v>
       </c>
     </row>
-    <row r="7" spans="1:5" ht="68">
+    <row r="7" spans="1:6" ht="68">
       <c r="A7" s="116" t="s">
         <v>202</v>
       </c>
@@ -9885,7 +9882,7 @@
         <v>1160</v>
       </c>
     </row>
-    <row r="8" spans="1:5" ht="91.5" customHeight="1">
+    <row r="8" spans="1:6" ht="91.5" customHeight="1">
       <c r="A8" s="116" t="s">
         <v>203</v>
       </c>
@@ -9902,7 +9899,7 @@
         <v>1157</v>
       </c>
     </row>
-    <row r="9" spans="1:5" ht="102">
+    <row r="9" spans="1:6" ht="102">
       <c r="A9" s="116" t="s">
         <v>203</v>
       </c>
@@ -9919,7 +9916,7 @@
         <v>1154</v>
       </c>
     </row>
-    <row r="10" spans="1:5" ht="51">
+    <row r="10" spans="1:6" ht="51">
       <c r="A10" s="116" t="s">
         <v>203</v>
       </c>
@@ -9936,7 +9933,7 @@
         <v>1151</v>
       </c>
     </row>
-    <row r="11" spans="1:5" ht="68">
+    <row r="11" spans="1:6" ht="68">
       <c r="A11" s="116" t="s">
         <v>204</v>
       </c>
@@ -9953,7 +9950,7 @@
         <v>1148</v>
       </c>
     </row>
-    <row r="12" spans="1:5" ht="102">
+    <row r="12" spans="1:6" ht="102">
       <c r="A12" s="116" t="s">
         <v>204</v>
       </c>
@@ -9970,7 +9967,7 @@
         <v>1145</v>
       </c>
     </row>
-    <row r="13" spans="1:5" ht="68">
+    <row r="13" spans="1:6" ht="68">
       <c r="A13" s="116" t="s">
         <v>204</v>
       </c>
@@ -9987,7 +9984,7 @@
         <v>1142</v>
       </c>
     </row>
-    <row r="14" spans="1:5" ht="68">
+    <row r="14" spans="1:6" ht="68">
       <c r="A14" s="116" t="s">
         <v>204</v>
       </c>
@@ -10004,7 +10001,7 @@
         <v>1139</v>
       </c>
     </row>
-    <row r="15" spans="1:5" ht="85">
+    <row r="15" spans="1:6" ht="85">
       <c r="A15" s="116" t="s">
         <v>204</v>
       </c>
@@ -10021,7 +10018,7 @@
         <v>1136</v>
       </c>
     </row>
-    <row r="16" spans="1:5" ht="68">
+    <row r="16" spans="1:6" ht="68">
       <c r="A16" s="116" t="s">
         <v>204</v>
       </c>
@@ -10123,7 +10120,7 @@
         <v>1118</v>
       </c>
     </row>
-    <row r="22" spans="1:5" ht="51">
+    <row r="22" spans="1:5" ht="68">
       <c r="A22" s="116" t="s">
         <v>205</v>
       </c>
@@ -10257,6 +10254,9 @@
       <c r="E1" t="s">
         <v>1049</v>
       </c>
+      <c r="F1" s="108" t="s">
+        <v>1478</v>
+      </c>
     </row>
     <row r="2" spans="1:21" ht="111" customHeight="1">
       <c r="A2" s="72" t="s">
@@ -13643,17 +13643,17 @@
 
 <file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B5344526-0759-5748-9599-6774FD0E2E70}">
-  <dimension ref="A1:E27"/>
+  <dimension ref="A1:F27"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="11.5" defaultRowHeight="16"/>
   <cols>
     <col min="1" max="1" width="65.1640625" customWidth="1"/>
     <col min="2" max="2" width="10" customWidth="1"/>
     <col min="3" max="3" width="134.5" customWidth="1"/>
     <col min="4" max="4" width="42.33203125" customWidth="1"/>
-    <col min="5" max="5" width="55" style="132" customWidth="1"/>
+    <col min="5" max="5" width="55" style="133" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5">
+    <row r="1" spans="1:6">
       <c r="A1" t="s">
         <v>199</v>
       </c>
@@ -13669,446 +13669,449 @@
       <c r="E1" t="s">
         <v>1058</v>
       </c>
-    </row>
-    <row r="2" spans="1:5" s="34" customFormat="1" ht="19">
-      <c r="A2" s="135" t="s">
+      <c r="F1" s="108" t="s">
+        <v>1479</v>
+      </c>
+    </row>
+    <row r="2" spans="1:6" s="34" customFormat="1" ht="19">
+      <c r="A2" s="136" t="s">
         <v>1356</v>
       </c>
       <c r="B2" s="33">
         <v>1</v>
       </c>
-      <c r="C2" s="133" t="s">
+      <c r="C2" s="134" t="s">
         <v>1371</v>
       </c>
-      <c r="D2" s="133" t="s">
+      <c r="D2" s="134" t="s">
         <v>1370</v>
       </c>
-      <c r="E2" s="133" t="s">
+      <c r="E2" s="134" t="s">
         <v>1369</v>
       </c>
     </row>
-    <row r="3" spans="1:5" ht="19">
-      <c r="A3" s="135" t="s">
+    <row r="3" spans="1:6" ht="19">
+      <c r="A3" s="136" t="s">
         <v>1356</v>
       </c>
       <c r="B3" s="33">
         <v>2</v>
       </c>
-      <c r="C3" s="136" t="s">
+      <c r="C3" s="137" t="s">
         <v>1368</v>
       </c>
-      <c r="D3" s="133" t="s">
+      <c r="D3" s="134" t="s">
         <v>1367</v>
       </c>
-      <c r="E3" s="133" t="s">
+      <c r="E3" s="134" t="s">
         <v>1366</v>
       </c>
     </row>
-    <row r="4" spans="1:5" ht="19">
-      <c r="A4" s="135" t="s">
+    <row r="4" spans="1:6" ht="19">
+      <c r="A4" s="136" t="s">
         <v>1356</v>
       </c>
       <c r="B4" s="33">
         <v>3</v>
       </c>
-      <c r="C4" s="134" t="s">
+      <c r="C4" s="135" t="s">
         <v>1365</v>
       </c>
-      <c r="D4" s="133" t="s">
+      <c r="D4" s="134" t="s">
         <v>1364</v>
       </c>
-      <c r="E4" s="133" t="s">
+      <c r="E4" s="134" t="s">
         <v>1363</v>
       </c>
     </row>
-    <row r="5" spans="1:5" ht="19">
-      <c r="A5" s="135" t="s">
+    <row r="5" spans="1:6" ht="19">
+      <c r="A5" s="136" t="s">
         <v>1356</v>
       </c>
       <c r="B5" s="31">
         <v>4</v>
       </c>
-      <c r="C5" s="134" t="s">
+      <c r="C5" s="135" t="s">
         <v>1362</v>
       </c>
-      <c r="D5" s="133" t="s">
+      <c r="D5" s="134" t="s">
         <v>1361</v>
       </c>
-      <c r="E5" s="133" t="s">
+      <c r="E5" s="134" t="s">
         <v>1360</v>
       </c>
     </row>
-    <row r="6" spans="1:5" ht="19">
-      <c r="A6" s="135" t="s">
+    <row r="6" spans="1:6" ht="19">
+      <c r="A6" s="136" t="s">
         <v>1356</v>
       </c>
       <c r="B6" s="31">
         <v>5</v>
       </c>
-      <c r="C6" s="134" t="s">
+      <c r="C6" s="135" t="s">
         <v>1359</v>
       </c>
-      <c r="D6" s="133" t="s">
+      <c r="D6" s="134" t="s">
         <v>1358</v>
       </c>
-      <c r="E6" s="133" t="s">
+      <c r="E6" s="134" t="s">
         <v>1357</v>
       </c>
     </row>
-    <row r="7" spans="1:5" ht="19">
-      <c r="A7" s="135" t="s">
+    <row r="7" spans="1:6" ht="19">
+      <c r="A7" s="136" t="s">
         <v>1356</v>
       </c>
       <c r="B7" s="31">
         <v>6</v>
       </c>
-      <c r="C7" s="134" t="s">
+      <c r="C7" s="135" t="s">
         <v>1355</v>
       </c>
-      <c r="D7" s="133" t="s">
+      <c r="D7" s="134" t="s">
         <v>1354</v>
       </c>
-      <c r="E7" s="133" t="s">
+      <c r="E7" s="134" t="s">
         <v>1353</v>
       </c>
     </row>
-    <row r="8" spans="1:5" ht="19">
-      <c r="A8" s="135" t="s">
+    <row r="8" spans="1:6" ht="19">
+      <c r="A8" s="136" t="s">
         <v>1347</v>
       </c>
       <c r="B8" s="31">
         <v>7</v>
       </c>
-      <c r="C8" s="134" t="s">
+      <c r="C8" s="135" t="s">
         <v>1352</v>
       </c>
-      <c r="D8" s="133" t="s">
+      <c r="D8" s="134" t="s">
         <v>1351</v>
       </c>
-      <c r="E8" s="133" t="s">
+      <c r="E8" s="134" t="s">
         <v>1350</v>
       </c>
     </row>
-    <row r="9" spans="1:5" ht="19">
-      <c r="A9" s="135" t="s">
+    <row r="9" spans="1:6" ht="19">
+      <c r="A9" s="136" t="s">
         <v>1347</v>
       </c>
       <c r="B9" s="31">
         <v>8</v>
       </c>
-      <c r="C9" s="134" t="s">
+      <c r="C9" s="135" t="s">
         <v>1349</v>
       </c>
-      <c r="D9" s="133" t="s">
+      <c r="D9" s="134" t="s">
         <v>1349</v>
       </c>
-      <c r="E9" s="133" t="s">
+      <c r="E9" s="134" t="s">
         <v>1348</v>
       </c>
     </row>
-    <row r="10" spans="1:5" ht="19">
-      <c r="A10" s="135" t="s">
+    <row r="10" spans="1:6" ht="19">
+      <c r="A10" s="136" t="s">
         <v>1347</v>
       </c>
       <c r="B10" s="31">
         <v>9</v>
       </c>
-      <c r="C10" s="134" t="s">
+      <c r="C10" s="135" t="s">
         <v>1346</v>
       </c>
-      <c r="D10" s="133" t="s">
+      <c r="D10" s="134" t="s">
         <v>1346</v>
       </c>
-      <c r="E10" s="133" t="s">
+      <c r="E10" s="134" t="s">
         <v>1345</v>
       </c>
     </row>
-    <row r="11" spans="1:5" ht="19">
-      <c r="A11" s="135" t="s">
+    <row r="11" spans="1:6" ht="19">
+      <c r="A11" s="136" t="s">
         <v>1316</v>
       </c>
       <c r="B11" s="31">
         <v>10</v>
       </c>
-      <c r="C11" s="134" t="s">
+      <c r="C11" s="135" t="s">
         <v>1344</v>
       </c>
-      <c r="D11" s="133" t="s">
+      <c r="D11" s="134" t="s">
         <v>1343</v>
       </c>
-      <c r="E11" s="133" t="s">
+      <c r="E11" s="134" t="s">
         <v>1342</v>
       </c>
     </row>
-    <row r="12" spans="1:5">
-      <c r="A12" s="135" t="s">
+    <row r="12" spans="1:6">
+      <c r="A12" s="136" t="s">
         <v>1316</v>
       </c>
       <c r="B12" s="31">
         <v>11</v>
       </c>
-      <c r="C12" s="134" t="s">
+      <c r="C12" s="135" t="s">
         <v>1341</v>
       </c>
-      <c r="D12" s="133" t="s">
+      <c r="D12" s="134" t="s">
         <v>1340</v>
       </c>
-      <c r="E12" s="133" t="s">
+      <c r="E12" s="134" t="s">
         <v>1339</v>
       </c>
     </row>
-    <row r="13" spans="1:5" ht="19">
-      <c r="A13" s="135" t="s">
+    <row r="13" spans="1:6" ht="19">
+      <c r="A13" s="136" t="s">
         <v>1316</v>
       </c>
       <c r="B13" s="31">
         <v>12</v>
       </c>
-      <c r="C13" s="134" t="s">
+      <c r="C13" s="135" t="s">
         <v>1338</v>
       </c>
-      <c r="D13" s="133" t="s">
+      <c r="D13" s="134" t="s">
         <v>1337</v>
       </c>
-      <c r="E13" s="133" t="s">
+      <c r="E13" s="134" t="s">
         <v>1336</v>
       </c>
     </row>
-    <row r="14" spans="1:5" ht="20">
-      <c r="A14" s="135" t="s">
+    <row r="14" spans="1:6" ht="20">
+      <c r="A14" s="136" t="s">
         <v>1316</v>
       </c>
       <c r="B14" s="31">
         <v>13</v>
       </c>
-      <c r="C14" s="134" t="s">
+      <c r="C14" s="135" t="s">
         <v>1335</v>
       </c>
-      <c r="D14" s="133" t="s">
+      <c r="D14" s="134" t="s">
         <v>1334</v>
       </c>
-      <c r="E14" s="133" t="s">
+      <c r="E14" s="134" t="s">
         <v>1333</v>
       </c>
     </row>
-    <row r="15" spans="1:5">
-      <c r="A15" s="135" t="s">
+    <row r="15" spans="1:6">
+      <c r="A15" s="136" t="s">
         <v>1316</v>
       </c>
       <c r="B15" s="31">
         <v>14</v>
       </c>
-      <c r="C15" s="134" t="s">
+      <c r="C15" s="135" t="s">
         <v>1332</v>
       </c>
-      <c r="D15" s="133" t="s">
+      <c r="D15" s="134" t="s">
         <v>1331</v>
       </c>
-      <c r="E15" s="133" t="s">
+      <c r="E15" s="134" t="s">
         <v>1330</v>
       </c>
     </row>
-    <row r="16" spans="1:5" ht="19">
-      <c r="A16" s="135" t="s">
+    <row r="16" spans="1:6" ht="19">
+      <c r="A16" s="136" t="s">
         <v>1316</v>
       </c>
       <c r="B16" s="31">
         <v>15</v>
       </c>
-      <c r="C16" s="134" t="s">
+      <c r="C16" s="135" t="s">
         <v>1329</v>
       </c>
-      <c r="D16" s="133" t="s">
+      <c r="D16" s="134" t="s">
         <v>1328</v>
       </c>
-      <c r="E16" s="133" t="s">
+      <c r="E16" s="134" t="s">
         <v>1328</v>
       </c>
     </row>
     <row r="17" spans="1:5">
-      <c r="A17" s="135" t="s">
+      <c r="A17" s="136" t="s">
         <v>1316</v>
       </c>
       <c r="B17" s="31">
         <v>16</v>
       </c>
-      <c r="C17" s="134" t="s">
+      <c r="C17" s="135" t="s">
         <v>1327</v>
       </c>
-      <c r="D17" s="133" t="s">
+      <c r="D17" s="134" t="s">
         <v>1326</v>
       </c>
-      <c r="E17" s="133" t="s">
+      <c r="E17" s="134" t="s">
         <v>1326</v>
       </c>
     </row>
     <row r="18" spans="1:5" ht="19">
-      <c r="A18" s="135" t="s">
+      <c r="A18" s="136" t="s">
         <v>1316</v>
       </c>
       <c r="B18" s="31">
         <v>17</v>
       </c>
-      <c r="C18" s="134" t="s">
+      <c r="C18" s="135" t="s">
         <v>1325</v>
       </c>
-      <c r="D18" s="133" t="s">
+      <c r="D18" s="134" t="s">
         <v>1324</v>
       </c>
-      <c r="E18" s="133" t="s">
+      <c r="E18" s="134" t="s">
         <v>1323</v>
       </c>
     </row>
     <row r="19" spans="1:5" ht="19">
-      <c r="A19" s="135" t="s">
+      <c r="A19" s="136" t="s">
         <v>1316</v>
       </c>
       <c r="B19" s="31">
         <v>18</v>
       </c>
-      <c r="C19" s="134" t="s">
+      <c r="C19" s="135" t="s">
         <v>1322</v>
       </c>
-      <c r="D19" s="133" t="s">
+      <c r="D19" s="134" t="s">
         <v>1321</v>
       </c>
-      <c r="E19" s="133" t="s">
+      <c r="E19" s="134" t="s">
         <v>1320</v>
       </c>
     </row>
     <row r="20" spans="1:5" ht="19">
-      <c r="A20" s="135" t="s">
+      <c r="A20" s="136" t="s">
         <v>1316</v>
       </c>
       <c r="B20" s="31">
         <v>19</v>
       </c>
-      <c r="C20" s="134" t="s">
+      <c r="C20" s="135" t="s">
         <v>1319</v>
       </c>
-      <c r="D20" s="133" t="s">
+      <c r="D20" s="134" t="s">
         <v>1318</v>
       </c>
-      <c r="E20" s="133" t="s">
+      <c r="E20" s="134" t="s">
         <v>1317</v>
       </c>
     </row>
     <row r="21" spans="1:5">
-      <c r="A21" s="135" t="s">
+      <c r="A21" s="136" t="s">
         <v>1316</v>
       </c>
       <c r="B21" s="31">
         <v>20</v>
       </c>
-      <c r="C21" s="134" t="s">
+      <c r="C21" s="135" t="s">
         <v>1315</v>
       </c>
-      <c r="D21" s="133" t="s">
+      <c r="D21" s="134" t="s">
         <v>1314</v>
       </c>
-      <c r="E21" s="133" t="s">
+      <c r="E21" s="134" t="s">
         <v>1313</v>
       </c>
     </row>
     <row r="22" spans="1:5" ht="19">
-      <c r="A22" s="135" t="s">
+      <c r="A22" s="136" t="s">
         <v>1306</v>
       </c>
       <c r="B22" s="31">
         <v>21</v>
       </c>
-      <c r="C22" s="134" t="s">
+      <c r="C22" s="135" t="s">
         <v>1312</v>
       </c>
-      <c r="D22" s="133" t="s">
+      <c r="D22" s="134" t="s">
         <v>1311</v>
       </c>
-      <c r="E22" s="133" t="s">
+      <c r="E22" s="134" t="s">
         <v>1310</v>
       </c>
     </row>
     <row r="23" spans="1:5" ht="19">
-      <c r="A23" s="135" t="s">
+      <c r="A23" s="136" t="s">
         <v>1306</v>
       </c>
       <c r="B23" s="31">
         <v>22</v>
       </c>
-      <c r="C23" s="134" t="s">
+      <c r="C23" s="135" t="s">
         <v>1309</v>
       </c>
-      <c r="D23" s="133" t="s">
+      <c r="D23" s="134" t="s">
         <v>1308</v>
       </c>
-      <c r="E23" s="133" t="s">
+      <c r="E23" s="134" t="s">
         <v>1307</v>
       </c>
     </row>
     <row r="24" spans="1:5" ht="19">
-      <c r="A24" s="135" t="s">
+      <c r="A24" s="136" t="s">
         <v>1306</v>
       </c>
       <c r="B24" s="31">
         <v>23</v>
       </c>
-      <c r="C24" s="134" t="s">
+      <c r="C24" s="135" t="s">
         <v>1305</v>
       </c>
-      <c r="D24" s="133" t="s">
+      <c r="D24" s="134" t="s">
         <v>1304</v>
       </c>
-      <c r="E24" s="133" t="s">
+      <c r="E24" s="134" t="s">
         <v>1303</v>
       </c>
     </row>
     <row r="25" spans="1:5" ht="19">
-      <c r="A25" s="135" t="s">
+      <c r="A25" s="136" t="s">
         <v>1295</v>
       </c>
       <c r="B25" s="31">
         <v>24</v>
       </c>
-      <c r="C25" s="134" t="s">
+      <c r="C25" s="135" t="s">
         <v>1302</v>
       </c>
-      <c r="D25" s="133" t="s">
+      <c r="D25" s="134" t="s">
         <v>1301</v>
       </c>
-      <c r="E25" s="133" t="s">
+      <c r="E25" s="134" t="s">
         <v>1300</v>
       </c>
     </row>
     <row r="26" spans="1:5" ht="19">
-      <c r="A26" s="135" t="s">
+      <c r="A26" s="136" t="s">
         <v>1299</v>
       </c>
       <c r="B26" s="31">
         <v>25</v>
       </c>
-      <c r="C26" s="134" t="s">
+      <c r="C26" s="135" t="s">
         <v>1298</v>
       </c>
-      <c r="D26" s="133" t="s">
+      <c r="D26" s="134" t="s">
         <v>1297</v>
       </c>
-      <c r="E26" s="133" t="s">
+      <c r="E26" s="134" t="s">
         <v>1296</v>
       </c>
     </row>
     <row r="27" spans="1:5" ht="20" thickBot="1">
-      <c r="A27" s="135" t="s">
+      <c r="A27" s="136" t="s">
         <v>1295</v>
       </c>
       <c r="B27" s="28">
         <v>26</v>
       </c>
-      <c r="C27" s="134" t="s">
+      <c r="C27" s="135" t="s">
         <v>1294</v>
       </c>
-      <c r="D27" s="133" t="s">
+      <c r="D27" s="134" t="s">
         <v>1293</v>
       </c>
-      <c r="E27" s="133" t="s">
+      <c r="E27" s="134" t="s">
         <v>1292</v>
       </c>
     </row>
@@ -14119,16 +14122,16 @@
 
 <file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{DD20F301-A307-714C-9879-0F7D8927DA0D}">
-  <dimension ref="A1:E27"/>
+  <dimension ref="A1:F27"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="11.5" defaultRowHeight="16"/>
   <cols>
     <col min="1" max="1" width="25.1640625" customWidth="1"/>
     <col min="2" max="2" width="10" customWidth="1"/>
     <col min="3" max="4" width="42.33203125" customWidth="1"/>
-    <col min="5" max="5" width="42.33203125" style="132" customWidth="1"/>
+    <col min="5" max="5" width="42.33203125" style="133" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5">
+    <row r="1" spans="1:6">
       <c r="A1" t="s">
         <v>1060</v>
       </c>
@@ -14144,8 +14147,11 @@
       <c r="E1" t="s">
         <v>1064</v>
       </c>
-    </row>
-    <row r="2" spans="1:5" s="34" customFormat="1" ht="68">
+      <c r="F1" s="108" t="s">
+        <v>1480</v>
+      </c>
+    </row>
+    <row r="2" spans="1:6" s="34" customFormat="1" ht="68">
       <c r="A2" s="23" t="s">
         <v>1453</v>
       </c>
@@ -14162,7 +14168,7 @@
         <v>1466</v>
       </c>
     </row>
-    <row r="3" spans="1:5" ht="68">
+    <row r="3" spans="1:6" ht="68">
       <c r="A3" s="23" t="s">
         <v>1453</v>
       </c>
@@ -14179,7 +14185,7 @@
         <v>1463</v>
       </c>
     </row>
-    <row r="4" spans="1:5" ht="102">
+    <row r="4" spans="1:6" ht="102">
       <c r="A4" s="23" t="s">
         <v>1453</v>
       </c>
@@ -14196,7 +14202,7 @@
         <v>1460</v>
       </c>
     </row>
-    <row r="5" spans="1:5" ht="102">
+    <row r="5" spans="1:6" ht="102">
       <c r="A5" s="23" t="s">
         <v>1453</v>
       </c>
@@ -14213,7 +14219,7 @@
         <v>1457</v>
       </c>
     </row>
-    <row r="6" spans="1:5" ht="102">
+    <row r="6" spans="1:6" ht="102">
       <c r="A6" s="23" t="s">
         <v>1453</v>
       </c>
@@ -14230,7 +14236,7 @@
         <v>1454</v>
       </c>
     </row>
-    <row r="7" spans="1:5" ht="57">
+    <row r="7" spans="1:6" ht="57">
       <c r="A7" s="23" t="s">
         <v>1453</v>
       </c>
@@ -14247,7 +14253,7 @@
         <v>1450</v>
       </c>
     </row>
-    <row r="8" spans="1:5" ht="68">
+    <row r="8" spans="1:6" ht="68">
       <c r="A8" s="23" t="s">
         <v>1443</v>
       </c>
@@ -14264,7 +14270,7 @@
         <v>1447</v>
       </c>
     </row>
-    <row r="9" spans="1:5" ht="85">
+    <row r="9" spans="1:6" ht="85">
       <c r="A9" s="23" t="s">
         <v>1443</v>
       </c>
@@ -14281,7 +14287,7 @@
         <v>1444</v>
       </c>
     </row>
-    <row r="10" spans="1:5" ht="38">
+    <row r="10" spans="1:6" ht="38">
       <c r="A10" s="23" t="s">
         <v>1443</v>
       </c>
@@ -14298,7 +14304,7 @@
         <v>1440</v>
       </c>
     </row>
-    <row r="11" spans="1:5" ht="51">
+    <row r="11" spans="1:6" ht="51">
       <c r="A11" s="23" t="s">
         <v>1409</v>
       </c>
@@ -14315,7 +14321,7 @@
         <v>1437</v>
       </c>
     </row>
-    <row r="12" spans="1:5" ht="85">
+    <row r="12" spans="1:6" ht="85">
       <c r="A12" s="23" t="s">
         <v>1409</v>
       </c>
@@ -14332,7 +14338,7 @@
         <v>1434</v>
       </c>
     </row>
-    <row r="13" spans="1:5" ht="57">
+    <row r="13" spans="1:6" ht="57">
       <c r="A13" s="23" t="s">
         <v>1409</v>
       </c>
@@ -14349,7 +14355,7 @@
         <v>1431</v>
       </c>
     </row>
-    <row r="14" spans="1:5" ht="57">
+    <row r="14" spans="1:6" ht="57">
       <c r="A14" s="23" t="s">
         <v>1409</v>
       </c>
@@ -14366,7 +14372,7 @@
         <v>1428</v>
       </c>
     </row>
-    <row r="15" spans="1:5" ht="76">
+    <row r="15" spans="1:6" ht="76">
       <c r="A15" s="23" t="s">
         <v>1409</v>
       </c>
@@ -14383,7 +14389,7 @@
         <v>1425</v>
       </c>
     </row>
-    <row r="16" spans="1:5" ht="51">
+    <row r="16" spans="1:6" ht="51">
       <c r="A16" s="23" t="s">
         <v>1409</v>
       </c>
@@ -14400,7 +14406,7 @@
         <v>1422</v>
       </c>
     </row>
-    <row r="17" spans="1:5" ht="51">
+    <row r="17" spans="1:5" ht="68">
       <c r="A17" s="23" t="s">
         <v>1409</v>
       </c>
@@ -14485,7 +14491,7 @@
         <v>1406</v>
       </c>
     </row>
-    <row r="22" spans="1:5" ht="51">
+    <row r="22" spans="1:5" ht="57">
       <c r="A22" s="23" t="s">
         <v>1399</v>
       </c>
@@ -14678,7 +14684,7 @@
       <c r="K2" s="72" t="s">
         <v>1178</v>
       </c>
-      <c r="L2" s="131" t="s">
+      <c r="L2" s="132" t="s">
         <v>1287</v>
       </c>
       <c r="M2" s="23" t="s">
@@ -14719,7 +14725,7 @@
       <c r="K3" s="72" t="s">
         <v>1179</v>
       </c>
-      <c r="L3" s="131" t="s">
+      <c r="L3" s="132" t="s">
         <v>1288</v>
       </c>
       <c r="M3" s="23" t="s">
@@ -14760,7 +14766,7 @@
       <c r="K4" s="72" t="s">
         <v>1180</v>
       </c>
-      <c r="L4" s="131" t="s">
+      <c r="L4" s="132" t="s">
         <v>1289</v>
       </c>
       <c r="M4" s="23" t="s">
@@ -14801,7 +14807,7 @@
       <c r="K5" s="72" t="s">
         <v>1181</v>
       </c>
-      <c r="L5" s="131" t="s">
+      <c r="L5" s="132" t="s">
         <v>1290</v>
       </c>
       <c r="M5" s="23" t="s">
@@ -14842,7 +14848,7 @@
       <c r="K6" s="72" t="s">
         <v>1182</v>
       </c>
-      <c r="L6" s="131" t="s">
+      <c r="L6" s="132" t="s">
         <v>1291</v>
       </c>
       <c r="M6" s="23" t="s">
@@ -14856,7 +14862,7 @@
 
 <file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2D128F0C-3C92-B24F-9D24-BF419F807E89}">
-  <dimension ref="A1:G49"/>
+  <dimension ref="A1:G44"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16"/>
   <cols>
     <col min="5" max="5" width="24.83203125" customWidth="1"/>
@@ -14891,10 +14897,10 @@
         <v>160</v>
       </c>
       <c r="B2" s="22" t="s">
+        <v>587</v>
+      </c>
+      <c r="C2" s="22" t="s">
         <v>588</v>
-      </c>
-      <c r="C2" s="22" t="s">
-        <v>587</v>
       </c>
       <c r="D2" s="22" t="s">
         <v>428</v>
@@ -14909,803 +14915,803 @@
         <v>590</v>
       </c>
     </row>
-    <row r="3" spans="1:7" ht="34">
+    <row r="3" spans="1:7">
       <c r="A3" t="s">
-        <v>160</v>
-      </c>
-      <c r="B3" s="22" t="s">
-        <v>1065</v>
-      </c>
-      <c r="C3" s="22" t="s">
-        <v>1066</v>
-      </c>
-      <c r="D3" s="22" t="s">
-        <v>428</v>
-      </c>
-      <c r="E3" s="46" t="s">
-        <v>1481</v>
-      </c>
-      <c r="F3" s="7" t="s">
-        <v>1470</v>
-      </c>
-      <c r="G3" s="22" t="s">
-        <v>1069</v>
+        <v>302</v>
+      </c>
+      <c r="B3" s="20" t="s">
+        <v>304</v>
+      </c>
+      <c r="C3" s="20" t="s">
+        <v>305</v>
+      </c>
+      <c r="D3" s="20" t="s">
+        <v>306</v>
+      </c>
+      <c r="E3" s="21" t="s">
+        <v>307</v>
+      </c>
+      <c r="F3" s="20" t="s">
+        <v>308</v>
+      </c>
+      <c r="G3" s="21" t="s">
+        <v>309</v>
       </c>
     </row>
     <row r="4" spans="1:7">
       <c r="A4" t="s">
-        <v>160</v>
-      </c>
-      <c r="B4" s="22" t="s">
-        <v>447</v>
-      </c>
-      <c r="C4" s="22" t="s">
-        <v>448</v>
-      </c>
-      <c r="D4" s="22" t="s">
-        <v>428</v>
-      </c>
-      <c r="E4" s="46" t="s">
-        <v>449</v>
-      </c>
-      <c r="F4" s="22" t="s">
-        <v>450</v>
-      </c>
-      <c r="G4" s="22" t="s">
-        <v>451</v>
+        <v>302</v>
+      </c>
+      <c r="B4" s="20" t="s">
+        <v>310</v>
+      </c>
+      <c r="C4" s="20" t="s">
+        <v>311</v>
+      </c>
+      <c r="D4" s="20" t="s">
+        <v>312</v>
+      </c>
+      <c r="E4" s="21" t="s">
+        <v>313</v>
+      </c>
+      <c r="F4" s="20" t="s">
+        <v>314</v>
+      </c>
+      <c r="G4" s="21" t="s">
+        <v>315</v>
       </c>
     </row>
     <row r="5" spans="1:7">
       <c r="A5" t="s">
-        <v>160</v>
-      </c>
-      <c r="B5" s="22" t="s">
-        <v>1476</v>
-      </c>
-      <c r="C5" s="22" t="s">
-        <v>1090</v>
-      </c>
-      <c r="D5" s="22" t="s">
-        <v>428</v>
-      </c>
-      <c r="E5" s="46" t="s">
-        <v>1091</v>
-      </c>
-      <c r="F5" t="s">
-        <v>1471</v>
-      </c>
-      <c r="G5" s="22" t="s">
-        <v>1094</v>
+        <v>302</v>
+      </c>
+      <c r="B5" s="20" t="s">
+        <v>316</v>
+      </c>
+      <c r="C5" s="20" t="s">
+        <v>317</v>
+      </c>
+      <c r="D5" s="20" t="s">
+        <v>318</v>
+      </c>
+      <c r="E5" s="21" t="s">
+        <v>319</v>
+      </c>
+      <c r="F5" s="20" t="s">
+        <v>314</v>
+      </c>
+      <c r="G5" s="21" t="s">
+        <v>320</v>
       </c>
     </row>
     <row r="6" spans="1:7">
       <c r="A6" t="s">
-        <v>160</v>
-      </c>
-      <c r="B6" s="22" t="s">
-        <v>1478</v>
-      </c>
-      <c r="C6" s="22" t="s">
-        <v>1477</v>
-      </c>
-      <c r="D6" s="22" t="s">
-        <v>428</v>
-      </c>
-      <c r="E6" s="46" t="s">
-        <v>1480</v>
-      </c>
-      <c r="F6" t="s">
-        <v>1472</v>
-      </c>
-      <c r="G6" s="22" t="s">
-        <v>1482</v>
+        <v>302</v>
+      </c>
+      <c r="B6" s="20" t="s">
+        <v>321</v>
+      </c>
+      <c r="C6" s="20" t="s">
+        <v>322</v>
+      </c>
+      <c r="D6" s="20" t="s">
+        <v>306</v>
+      </c>
+      <c r="E6" s="21" t="s">
+        <v>323</v>
+      </c>
+      <c r="F6" s="20" t="s">
+        <v>324</v>
+      </c>
+      <c r="G6" s="21" t="s">
+        <v>325</v>
       </c>
     </row>
     <row r="7" spans="1:7">
       <c r="A7" t="s">
-        <v>160</v>
-      </c>
-      <c r="B7" s="22" t="s">
-        <v>1475</v>
-      </c>
-      <c r="C7" s="22" t="s">
-        <v>1474</v>
-      </c>
-      <c r="D7" s="22" t="s">
-        <v>428</v>
-      </c>
-      <c r="E7" s="46" t="s">
-        <v>1479</v>
-      </c>
-      <c r="F7" t="s">
-        <v>1473</v>
-      </c>
-      <c r="G7" s="22" t="s">
-        <v>1483</v>
+        <v>337</v>
+      </c>
+      <c r="B7" s="35" t="s">
+        <v>421</v>
+      </c>
+      <c r="C7" s="35" t="s">
+        <v>422</v>
+      </c>
+      <c r="D7" s="35" t="s">
+        <v>423</v>
+      </c>
+      <c r="E7" s="36" t="s">
+        <v>424</v>
+      </c>
+      <c r="F7" s="35" t="s">
+        <v>425</v>
+      </c>
+      <c r="G7" s="37" t="s">
+        <v>798</v>
       </c>
     </row>
     <row r="8" spans="1:7">
       <c r="A8" t="s">
-        <v>302</v>
-      </c>
-      <c r="B8" s="20" t="s">
-        <v>304</v>
-      </c>
-      <c r="C8" s="20" t="s">
-        <v>305</v>
-      </c>
-      <c r="D8" s="20" t="s">
-        <v>306</v>
-      </c>
-      <c r="E8" s="21" t="s">
-        <v>307</v>
-      </c>
-      <c r="F8" s="20" t="s">
-        <v>308</v>
-      </c>
-      <c r="G8" s="21" t="s">
-        <v>309</v>
+        <v>337</v>
+      </c>
+      <c r="B8" s="35" t="s">
+        <v>426</v>
+      </c>
+      <c r="C8" s="35" t="s">
+        <v>427</v>
+      </c>
+      <c r="D8" s="35" t="s">
+        <v>428</v>
+      </c>
+      <c r="E8" s="36" t="s">
+        <v>429</v>
+      </c>
+      <c r="F8" s="35" t="s">
+        <v>430</v>
+      </c>
+      <c r="G8" s="37" t="s">
+        <v>797</v>
       </c>
     </row>
     <row r="9" spans="1:7">
       <c r="A9" t="s">
-        <v>302</v>
-      </c>
-      <c r="B9" s="20" t="s">
-        <v>310</v>
-      </c>
-      <c r="C9" s="20" t="s">
-        <v>311</v>
-      </c>
-      <c r="D9" s="20" t="s">
-        <v>312</v>
-      </c>
-      <c r="E9" s="21" t="s">
-        <v>313</v>
-      </c>
-      <c r="F9" s="20" t="s">
-        <v>314</v>
-      </c>
-      <c r="G9" s="21" t="s">
-        <v>315</v>
-      </c>
+        <v>337</v>
+      </c>
+      <c r="B9" s="35" t="s">
+        <v>431</v>
+      </c>
+      <c r="C9" s="35" t="s">
+        <v>432</v>
+      </c>
+      <c r="D9" s="35" t="s">
+        <v>433</v>
+      </c>
+      <c r="E9" s="35" t="s">
+        <v>434</v>
+      </c>
+      <c r="F9" s="35" t="s">
+        <v>435</v>
+      </c>
+      <c r="G9" s="38"/>
     </row>
     <row r="10" spans="1:7">
       <c r="A10" t="s">
-        <v>302</v>
-      </c>
-      <c r="B10" s="20" t="s">
-        <v>316</v>
-      </c>
-      <c r="C10" s="20" t="s">
-        <v>317</v>
-      </c>
-      <c r="D10" s="20" t="s">
-        <v>318</v>
-      </c>
-      <c r="E10" s="21" t="s">
-        <v>319</v>
-      </c>
-      <c r="F10" s="20" t="s">
-        <v>314</v>
-      </c>
-      <c r="G10" s="21" t="s">
-        <v>320</v>
+        <v>214</v>
+      </c>
+      <c r="B10" t="s">
+        <v>436</v>
+      </c>
+      <c r="C10" t="s">
+        <v>437</v>
+      </c>
+      <c r="D10" t="s">
+        <v>799</v>
+      </c>
+      <c r="E10" t="s">
+        <v>438</v>
+      </c>
+      <c r="F10" t="s">
+        <v>439</v>
+      </c>
+      <c r="G10" t="s">
+        <v>440</v>
       </c>
     </row>
     <row r="11" spans="1:7">
       <c r="A11" t="s">
-        <v>302</v>
-      </c>
-      <c r="B11" s="20" t="s">
-        <v>321</v>
-      </c>
-      <c r="C11" s="20" t="s">
-        <v>322</v>
-      </c>
-      <c r="D11" s="20" t="s">
-        <v>306</v>
-      </c>
-      <c r="E11" s="21" t="s">
-        <v>323</v>
-      </c>
-      <c r="F11" s="20" t="s">
-        <v>324</v>
-      </c>
-      <c r="G11" s="21" t="s">
-        <v>325</v>
+        <v>214</v>
+      </c>
+      <c r="B11" t="s">
+        <v>441</v>
+      </c>
+      <c r="C11" t="s">
+        <v>442</v>
+      </c>
+      <c r="D11" t="s">
+        <v>443</v>
+      </c>
+      <c r="E11" t="s">
+        <v>444</v>
+      </c>
+      <c r="F11" t="s">
+        <v>445</v>
+      </c>
+      <c r="G11" t="s">
+        <v>446</v>
       </c>
     </row>
     <row r="12" spans="1:7">
       <c r="A12" t="s">
-        <v>337</v>
-      </c>
-      <c r="B12" s="35" t="s">
-        <v>421</v>
-      </c>
-      <c r="C12" s="35" t="s">
-        <v>422</v>
-      </c>
-      <c r="D12" s="35" t="s">
-        <v>423</v>
-      </c>
-      <c r="E12" s="36" t="s">
-        <v>424</v>
-      </c>
-      <c r="F12" s="35" t="s">
-        <v>425</v>
-      </c>
-      <c r="G12" s="37" t="s">
-        <v>798</v>
+        <v>214</v>
+      </c>
+      <c r="B12" t="s">
+        <v>447</v>
+      </c>
+      <c r="C12" t="s">
+        <v>448</v>
+      </c>
+      <c r="D12" t="s">
+        <v>428</v>
+      </c>
+      <c r="E12" t="s">
+        <v>449</v>
+      </c>
+      <c r="F12" t="s">
+        <v>450</v>
+      </c>
+      <c r="G12" t="s">
+        <v>451</v>
       </c>
     </row>
     <row r="13" spans="1:7">
       <c r="A13" t="s">
-        <v>337</v>
-      </c>
-      <c r="B13" s="35" t="s">
-        <v>426</v>
-      </c>
-      <c r="C13" s="35" t="s">
-        <v>427</v>
-      </c>
-      <c r="D13" s="35" t="s">
-        <v>428</v>
-      </c>
-      <c r="E13" s="36" t="s">
-        <v>429</v>
-      </c>
-      <c r="F13" s="35" t="s">
-        <v>430</v>
-      </c>
-      <c r="G13" s="37" t="s">
-        <v>797</v>
+        <v>214</v>
+      </c>
+      <c r="B13" t="s">
+        <v>452</v>
+      </c>
+      <c r="C13" t="s">
+        <v>453</v>
+      </c>
+      <c r="D13" t="s">
+        <v>454</v>
+      </c>
+      <c r="E13" t="s">
+        <v>455</v>
+      </c>
+      <c r="F13" t="s">
+        <v>456</v>
+      </c>
+      <c r="G13" t="s">
+        <v>457</v>
       </c>
     </row>
     <row r="14" spans="1:7">
       <c r="A14" t="s">
-        <v>337</v>
-      </c>
-      <c r="B14" s="35" t="s">
-        <v>431</v>
-      </c>
-      <c r="C14" s="35" t="s">
-        <v>432</v>
-      </c>
-      <c r="D14" s="35" t="s">
-        <v>433</v>
-      </c>
-      <c r="E14" s="35" t="s">
-        <v>434</v>
-      </c>
-      <c r="F14" s="35" t="s">
-        <v>435</v>
-      </c>
-      <c r="G14" s="38"/>
+        <v>214</v>
+      </c>
+      <c r="B14" t="s">
+        <v>458</v>
+      </c>
+      <c r="C14" t="s">
+        <v>459</v>
+      </c>
+      <c r="D14" t="s">
+        <v>460</v>
+      </c>
+      <c r="E14" t="s">
+        <v>461</v>
+      </c>
+      <c r="F14" t="s">
+        <v>462</v>
+      </c>
+      <c r="G14" t="s">
+        <v>463</v>
+      </c>
     </row>
     <row r="15" spans="1:7">
       <c r="A15" t="s">
         <v>214</v>
       </c>
       <c r="B15" t="s">
-        <v>436</v>
+        <v>464</v>
       </c>
       <c r="C15" t="s">
-        <v>437</v>
+        <v>465</v>
       </c>
       <c r="D15" t="s">
-        <v>799</v>
+        <v>466</v>
       </c>
       <c r="E15" t="s">
-        <v>438</v>
+        <v>467</v>
       </c>
       <c r="F15" t="s">
-        <v>439</v>
+        <v>468</v>
       </c>
       <c r="G15" t="s">
-        <v>440</v>
+        <v>469</v>
       </c>
     </row>
     <row r="16" spans="1:7">
       <c r="A16" t="s">
-        <v>214</v>
-      </c>
-      <c r="B16" t="s">
-        <v>441</v>
-      </c>
-      <c r="C16" t="s">
-        <v>442</v>
-      </c>
-      <c r="D16" t="s">
-        <v>443</v>
-      </c>
-      <c r="E16" t="s">
-        <v>444</v>
-      </c>
-      <c r="F16" t="s">
-        <v>445</v>
-      </c>
-      <c r="G16" t="s">
-        <v>446</v>
+        <v>554</v>
+      </c>
+      <c r="B16" s="49" t="s">
+        <v>562</v>
+      </c>
+      <c r="C16" s="47" t="s">
+        <v>563</v>
+      </c>
+      <c r="D16" s="47" t="s">
+        <v>564</v>
+      </c>
+      <c r="E16" s="46" t="s">
+        <v>555</v>
+      </c>
+      <c r="F16" s="47" t="s">
+        <v>556</v>
+      </c>
+      <c r="G16" s="48" t="s">
+        <v>557</v>
       </c>
     </row>
     <row r="17" spans="1:7">
       <c r="A17" t="s">
-        <v>214</v>
-      </c>
-      <c r="B17" t="s">
-        <v>447</v>
-      </c>
-      <c r="C17" t="s">
-        <v>448</v>
-      </c>
-      <c r="D17" t="s">
-        <v>428</v>
-      </c>
-      <c r="E17" t="s">
-        <v>449</v>
-      </c>
-      <c r="F17" t="s">
-        <v>450</v>
-      </c>
-      <c r="G17" t="s">
-        <v>451</v>
+        <v>554</v>
+      </c>
+      <c r="B17" s="49" t="s">
+        <v>565</v>
+      </c>
+      <c r="C17" s="47" t="s">
+        <v>566</v>
+      </c>
+      <c r="D17" s="47" t="s">
+        <v>567</v>
+      </c>
+      <c r="E17" s="48" t="s">
+        <v>558</v>
+      </c>
+      <c r="F17" s="47" t="s">
+        <v>556</v>
+      </c>
+      <c r="G17" s="48" t="s">
+        <v>559</v>
       </c>
     </row>
     <row r="18" spans="1:7">
       <c r="A18" t="s">
-        <v>214</v>
-      </c>
-      <c r="B18" t="s">
-        <v>452</v>
-      </c>
-      <c r="C18" t="s">
-        <v>453</v>
-      </c>
-      <c r="D18" t="s">
-        <v>454</v>
-      </c>
-      <c r="E18" t="s">
-        <v>455</v>
-      </c>
-      <c r="F18" t="s">
-        <v>456</v>
-      </c>
-      <c r="G18" t="s">
-        <v>457</v>
-      </c>
-    </row>
-    <row r="19" spans="1:7">
+        <v>554</v>
+      </c>
+      <c r="B18" s="49" t="s">
+        <v>568</v>
+      </c>
+      <c r="C18" s="47" t="s">
+        <v>569</v>
+      </c>
+      <c r="D18" s="47" t="s">
+        <v>567</v>
+      </c>
+      <c r="E18" s="48" t="s">
+        <v>560</v>
+      </c>
+      <c r="F18" s="47" t="s">
+        <v>556</v>
+      </c>
+      <c r="G18" s="47" t="s">
+        <v>561</v>
+      </c>
+    </row>
+    <row r="19" spans="1:7" ht="18">
       <c r="A19" t="s">
-        <v>214</v>
-      </c>
-      <c r="B19" t="s">
-        <v>458</v>
-      </c>
-      <c r="C19" t="s">
-        <v>459</v>
-      </c>
-      <c r="D19" t="s">
-        <v>460</v>
-      </c>
-      <c r="E19" t="s">
-        <v>461</v>
-      </c>
-      <c r="F19" t="s">
-        <v>462</v>
-      </c>
-      <c r="G19" t="s">
-        <v>463</v>
-      </c>
-    </row>
-    <row r="20" spans="1:7">
+        <v>586</v>
+      </c>
+      <c r="B19" s="49" t="s">
+        <v>570</v>
+      </c>
+      <c r="C19" s="49" t="s">
+        <v>571</v>
+      </c>
+      <c r="D19" s="49" t="s">
+        <v>306</v>
+      </c>
+      <c r="E19" s="50" t="s">
+        <v>572</v>
+      </c>
+      <c r="F19" s="49" t="s">
+        <v>573</v>
+      </c>
+      <c r="G19" s="46" t="s">
+        <v>593</v>
+      </c>
+    </row>
+    <row r="20" spans="1:7" ht="18">
       <c r="A20" t="s">
-        <v>214</v>
-      </c>
-      <c r="B20" t="s">
-        <v>464</v>
-      </c>
-      <c r="C20" t="s">
-        <v>465</v>
-      </c>
-      <c r="D20" t="s">
-        <v>466</v>
-      </c>
-      <c r="E20" t="s">
-        <v>467</v>
-      </c>
-      <c r="F20" t="s">
-        <v>468</v>
-      </c>
-      <c r="G20" t="s">
-        <v>469</v>
+        <v>586</v>
+      </c>
+      <c r="B20" s="49" t="s">
+        <v>574</v>
+      </c>
+      <c r="C20" s="49" t="s">
+        <v>575</v>
+      </c>
+      <c r="D20" s="49" t="s">
+        <v>306</v>
+      </c>
+      <c r="E20" s="50" t="s">
+        <v>576</v>
+      </c>
+      <c r="F20" s="49" t="s">
+        <v>577</v>
+      </c>
+      <c r="G20" s="46" t="s">
+        <v>592</v>
       </c>
     </row>
     <row r="21" spans="1:7">
       <c r="A21" t="s">
-        <v>554</v>
+        <v>586</v>
       </c>
       <c r="B21" s="49" t="s">
-        <v>562</v>
-      </c>
-      <c r="C21" s="47" t="s">
-        <v>563</v>
-      </c>
-      <c r="D21" s="47" t="s">
-        <v>564</v>
-      </c>
-      <c r="E21" s="46" t="s">
-        <v>555</v>
-      </c>
-      <c r="F21" s="47" t="s">
-        <v>556</v>
-      </c>
-      <c r="G21" s="48" t="s">
-        <v>557</v>
-      </c>
-    </row>
-    <row r="22" spans="1:7">
+        <v>578</v>
+      </c>
+      <c r="C21" s="49" t="s">
+        <v>579</v>
+      </c>
+      <c r="D21" s="49" t="s">
+        <v>306</v>
+      </c>
+      <c r="E21" s="49" t="s">
+        <v>580</v>
+      </c>
+      <c r="F21" s="49" t="s">
+        <v>581</v>
+      </c>
+      <c r="G21" s="46" t="s">
+        <v>591</v>
+      </c>
+    </row>
+    <row r="22" spans="1:7" ht="23">
       <c r="A22" t="s">
-        <v>554</v>
+        <v>586</v>
       </c>
       <c r="B22" s="49" t="s">
-        <v>565</v>
-      </c>
-      <c r="C22" s="47" t="s">
-        <v>566</v>
-      </c>
-      <c r="D22" s="47" t="s">
-        <v>567</v>
-      </c>
-      <c r="E22" s="48" t="s">
-        <v>558</v>
-      </c>
-      <c r="F22" s="47" t="s">
-        <v>556</v>
-      </c>
-      <c r="G22" s="48" t="s">
-        <v>559</v>
-      </c>
+        <v>578</v>
+      </c>
+      <c r="C22" s="49" t="s">
+        <v>582</v>
+      </c>
+      <c r="D22" s="49" t="s">
+        <v>583</v>
+      </c>
+      <c r="E22" s="46" t="s">
+        <v>584</v>
+      </c>
+      <c r="F22" s="49" t="s">
+        <v>585</v>
+      </c>
+      <c r="G22" s="51"/>
     </row>
     <row r="23" spans="1:7">
       <c r="A23" t="s">
-        <v>554</v>
-      </c>
-      <c r="B23" s="49" t="s">
-        <v>568</v>
-      </c>
-      <c r="C23" s="47" t="s">
-        <v>569</v>
-      </c>
-      <c r="D23" s="47" t="s">
-        <v>567</v>
-      </c>
-      <c r="E23" s="48" t="s">
-        <v>560</v>
-      </c>
-      <c r="F23" s="47" t="s">
-        <v>556</v>
-      </c>
-      <c r="G23" s="47" t="s">
-        <v>561</v>
-      </c>
-    </row>
-    <row r="24" spans="1:7" ht="18">
+        <v>775</v>
+      </c>
+      <c r="B23" s="80" t="s">
+        <v>776</v>
+      </c>
+      <c r="C23" s="80" t="s">
+        <v>777</v>
+      </c>
+      <c r="D23" s="80" t="s">
+        <v>778</v>
+      </c>
+      <c r="E23" s="80" t="s">
+        <v>779</v>
+      </c>
+      <c r="F23" s="80" t="s">
+        <v>780</v>
+      </c>
+      <c r="G23" s="88" t="s">
+        <v>793</v>
+      </c>
+    </row>
+    <row r="24" spans="1:7">
       <c r="A24" t="s">
-        <v>586</v>
-      </c>
-      <c r="B24" s="49" t="s">
-        <v>570</v>
-      </c>
-      <c r="C24" s="49" t="s">
-        <v>571</v>
-      </c>
-      <c r="D24" s="49" t="s">
-        <v>306</v>
-      </c>
-      <c r="E24" s="50" t="s">
-        <v>572</v>
-      </c>
-      <c r="F24" s="49" t="s">
-        <v>573</v>
-      </c>
-      <c r="G24" s="46" t="s">
-        <v>593</v>
-      </c>
-    </row>
-    <row r="25" spans="1:7" ht="18">
+        <v>775</v>
+      </c>
+      <c r="B24" s="80" t="s">
+        <v>781</v>
+      </c>
+      <c r="C24" s="80" t="s">
+        <v>782</v>
+      </c>
+      <c r="D24" s="80" t="s">
+        <v>318</v>
+      </c>
+      <c r="E24" s="82" t="s">
+        <v>783</v>
+      </c>
+      <c r="F24" s="83" t="s">
+        <v>784</v>
+      </c>
+      <c r="G24" s="89" t="s">
+        <v>794</v>
+      </c>
+    </row>
+    <row r="25" spans="1:7">
       <c r="A25" t="s">
-        <v>586</v>
-      </c>
-      <c r="B25" s="49" t="s">
-        <v>574</v>
-      </c>
-      <c r="C25" s="49" t="s">
-        <v>575</v>
-      </c>
-      <c r="D25" s="49" t="s">
-        <v>306</v>
-      </c>
-      <c r="E25" s="50" t="s">
-        <v>576</v>
-      </c>
-      <c r="F25" s="49" t="s">
-        <v>577</v>
-      </c>
-      <c r="G25" s="46" t="s">
-        <v>592</v>
+        <v>775</v>
+      </c>
+      <c r="B25" s="80" t="s">
+        <v>785</v>
+      </c>
+      <c r="C25" s="80" t="s">
+        <v>786</v>
+      </c>
+      <c r="D25" s="80" t="s">
+        <v>778</v>
+      </c>
+      <c r="E25" s="81" t="s">
+        <v>787</v>
+      </c>
+      <c r="F25" s="80" t="s">
+        <v>788</v>
+      </c>
+      <c r="G25" s="84" t="s">
+        <v>795</v>
       </c>
     </row>
     <row r="26" spans="1:7">
       <c r="A26" t="s">
-        <v>586</v>
-      </c>
-      <c r="B26" s="49" t="s">
-        <v>578</v>
-      </c>
-      <c r="C26" s="49" t="s">
-        <v>579</v>
-      </c>
-      <c r="D26" s="49" t="s">
-        <v>306</v>
-      </c>
-      <c r="E26" s="49" t="s">
-        <v>580</v>
-      </c>
-      <c r="F26" s="49" t="s">
-        <v>581</v>
-      </c>
-      <c r="G26" s="46" t="s">
-        <v>591</v>
-      </c>
-    </row>
-    <row r="27" spans="1:7" ht="23">
+        <v>775</v>
+      </c>
+      <c r="B26" s="85" t="s">
+        <v>789</v>
+      </c>
+      <c r="C26" s="80" t="s">
+        <v>790</v>
+      </c>
+      <c r="D26" s="24" t="s">
+        <v>428</v>
+      </c>
+      <c r="E26" s="86" t="s">
+        <v>791</v>
+      </c>
+      <c r="F26" s="87" t="s">
+        <v>792</v>
+      </c>
+      <c r="G26" s="81" t="s">
+        <v>796</v>
+      </c>
+    </row>
+    <row r="27" spans="1:7">
       <c r="A27" t="s">
-        <v>586</v>
+        <v>816</v>
       </c>
       <c r="B27" s="49" t="s">
-        <v>578</v>
+        <v>800</v>
       </c>
       <c r="C27" s="49" t="s">
-        <v>582</v>
+        <v>801</v>
       </c>
       <c r="D27" s="49" t="s">
-        <v>583</v>
+        <v>802</v>
       </c>
       <c r="E27" s="46" t="s">
-        <v>584</v>
+        <v>803</v>
       </c>
       <c r="F27" s="49" t="s">
-        <v>585</v>
-      </c>
-      <c r="G27" s="51"/>
+        <v>804</v>
+      </c>
+      <c r="G27" s="46" t="s">
+        <v>805</v>
+      </c>
     </row>
     <row r="28" spans="1:7">
       <c r="A28" t="s">
-        <v>775</v>
-      </c>
-      <c r="B28" s="80" t="s">
-        <v>776</v>
-      </c>
-      <c r="C28" s="80" t="s">
-        <v>777</v>
-      </c>
-      <c r="D28" s="80" t="s">
-        <v>778</v>
-      </c>
-      <c r="E28" s="80" t="s">
-        <v>779</v>
-      </c>
-      <c r="F28" s="80" t="s">
-        <v>780</v>
-      </c>
-      <c r="G28" s="88" t="s">
-        <v>793</v>
+        <v>816</v>
+      </c>
+      <c r="B28" s="49" t="s">
+        <v>806</v>
+      </c>
+      <c r="C28" s="49" t="s">
+        <v>807</v>
+      </c>
+      <c r="D28" s="49" t="s">
+        <v>428</v>
+      </c>
+      <c r="E28" s="46" t="s">
+        <v>808</v>
+      </c>
+      <c r="F28" s="49" t="s">
+        <v>809</v>
+      </c>
+      <c r="G28" s="46" t="s">
+        <v>810</v>
       </c>
     </row>
     <row r="29" spans="1:7">
       <c r="A29" t="s">
-        <v>775</v>
-      </c>
-      <c r="B29" s="80" t="s">
-        <v>781</v>
-      </c>
-      <c r="C29" s="80" t="s">
-        <v>782</v>
-      </c>
-      <c r="D29" s="80" t="s">
-        <v>318</v>
-      </c>
-      <c r="E29" s="82" t="s">
-        <v>783</v>
-      </c>
-      <c r="F29" s="83" t="s">
-        <v>784</v>
-      </c>
-      <c r="G29" s="89" t="s">
-        <v>794</v>
+        <v>816</v>
+      </c>
+      <c r="B29" s="49" t="s">
+        <v>811</v>
+      </c>
+      <c r="C29" s="49" t="s">
+        <v>812</v>
+      </c>
+      <c r="D29" s="49" t="s">
+        <v>428</v>
+      </c>
+      <c r="E29" s="46" t="s">
+        <v>813</v>
+      </c>
+      <c r="F29" s="49" t="s">
+        <v>814</v>
+      </c>
+      <c r="G29" s="49" t="s">
+        <v>815</v>
       </c>
     </row>
     <row r="30" spans="1:7">
       <c r="A30" t="s">
-        <v>775</v>
-      </c>
-      <c r="B30" s="80" t="s">
-        <v>785</v>
-      </c>
-      <c r="C30" s="80" t="s">
-        <v>786</v>
-      </c>
-      <c r="D30" s="80" t="s">
-        <v>778</v>
-      </c>
-      <c r="E30" s="81" t="s">
-        <v>787</v>
-      </c>
-      <c r="F30" s="80" t="s">
-        <v>788</v>
-      </c>
-      <c r="G30" s="84" t="s">
-        <v>795</v>
+        <v>993</v>
+      </c>
+      <c r="B30" s="49" t="s">
+        <v>994</v>
+      </c>
+      <c r="C30" s="49" t="s">
+        <v>995</v>
+      </c>
+      <c r="D30" s="49" t="s">
+        <v>996</v>
+      </c>
+      <c r="E30" s="46" t="s">
+        <v>997</v>
+      </c>
+      <c r="F30" s="49" t="s">
+        <v>998</v>
+      </c>
+      <c r="G30" s="49" t="s">
+        <v>999</v>
       </c>
     </row>
     <row r="31" spans="1:7">
       <c r="A31" t="s">
-        <v>775</v>
-      </c>
-      <c r="B31" s="85" t="s">
-        <v>789</v>
-      </c>
-      <c r="C31" s="80" t="s">
-        <v>790</v>
-      </c>
-      <c r="D31" s="24" t="s">
+        <v>993</v>
+      </c>
+      <c r="B31" s="49" t="s">
+        <v>1000</v>
+      </c>
+      <c r="C31" s="49" t="s">
+        <v>1001</v>
+      </c>
+      <c r="D31" s="49" t="s">
         <v>428</v>
       </c>
-      <c r="E31" s="86" t="s">
-        <v>791</v>
-      </c>
-      <c r="F31" s="87" t="s">
-        <v>792</v>
-      </c>
-      <c r="G31" s="81" t="s">
-        <v>796</v>
-      </c>
+      <c r="E31" s="46" t="s">
+        <v>1002</v>
+      </c>
+      <c r="F31" s="49" t="s">
+        <v>1003</v>
+      </c>
+      <c r="G31" s="46"/>
     </row>
     <row r="32" spans="1:7">
       <c r="A32" t="s">
-        <v>816</v>
+        <v>993</v>
       </c>
       <c r="B32" s="49" t="s">
-        <v>800</v>
+        <v>1004</v>
       </c>
       <c r="C32" s="49" t="s">
-        <v>801</v>
+        <v>1005</v>
       </c>
       <c r="D32" s="49" t="s">
-        <v>802</v>
+        <v>428</v>
       </c>
       <c r="E32" s="46" t="s">
-        <v>803</v>
+        <v>1006</v>
       </c>
       <c r="F32" s="49" t="s">
-        <v>804</v>
-      </c>
-      <c r="G32" s="46" t="s">
-        <v>805</v>
+        <v>1003</v>
+      </c>
+      <c r="G32" s="49" t="s">
+        <v>1007</v>
       </c>
     </row>
     <row r="33" spans="1:7">
       <c r="A33" t="s">
-        <v>816</v>
-      </c>
-      <c r="B33" s="49" t="s">
-        <v>806</v>
-      </c>
-      <c r="C33" s="49" t="s">
-        <v>807</v>
-      </c>
-      <c r="D33" s="49" t="s">
+        <v>1050</v>
+      </c>
+      <c r="B33" s="24" t="s">
+        <v>1065</v>
+      </c>
+      <c r="C33" s="24" t="s">
+        <v>1066</v>
+      </c>
+      <c r="D33" s="24" t="s">
         <v>428</v>
       </c>
-      <c r="E33" s="46" t="s">
-        <v>808</v>
-      </c>
-      <c r="F33" s="49" t="s">
-        <v>809</v>
-      </c>
-      <c r="G33" s="46" t="s">
-        <v>810</v>
+      <c r="E33" s="109" t="s">
+        <v>1067</v>
+      </c>
+      <c r="F33" s="24" t="s">
+        <v>1068</v>
+      </c>
+      <c r="G33" s="24" t="s">
+        <v>1069</v>
       </c>
     </row>
     <row r="34" spans="1:7">
       <c r="A34" t="s">
-        <v>816</v>
-      </c>
-      <c r="B34" s="49" t="s">
-        <v>811</v>
-      </c>
-      <c r="C34" s="49" t="s">
-        <v>812</v>
-      </c>
-      <c r="D34" s="49" t="s">
+        <v>1050</v>
+      </c>
+      <c r="B34" s="24" t="s">
+        <v>1070</v>
+      </c>
+      <c r="C34" s="24" t="s">
+        <v>1071</v>
+      </c>
+      <c r="D34" s="24" t="s">
         <v>428</v>
       </c>
-      <c r="E34" s="46" t="s">
-        <v>813</v>
-      </c>
-      <c r="F34" s="49" t="s">
-        <v>814</v>
-      </c>
-      <c r="G34" s="49" t="s">
-        <v>815</v>
+      <c r="E34" s="109" t="s">
+        <v>1072</v>
+      </c>
+      <c r="F34" s="24" t="s">
+        <v>1073</v>
+      </c>
+      <c r="G34" s="24" t="s">
+        <v>1074</v>
       </c>
     </row>
     <row r="35" spans="1:7">
       <c r="A35" t="s">
-        <v>993</v>
-      </c>
-      <c r="B35" s="49" t="s">
-        <v>994</v>
-      </c>
-      <c r="C35" s="49" t="s">
-        <v>995</v>
-      </c>
-      <c r="D35" s="49" t="s">
+        <v>1050</v>
+      </c>
+      <c r="B35" s="24" t="s">
+        <v>1075</v>
+      </c>
+      <c r="C35" s="24" t="s">
+        <v>1076</v>
+      </c>
+      <c r="D35" s="24" t="s">
         <v>996</v>
       </c>
-      <c r="E35" s="46" t="s">
-        <v>997</v>
-      </c>
-      <c r="F35" s="49" t="s">
-        <v>998</v>
-      </c>
-      <c r="G35" s="49" t="s">
-        <v>999</v>
+      <c r="E35" s="109" t="s">
+        <v>1077</v>
+      </c>
+      <c r="F35" s="24" t="s">
+        <v>1073</v>
+      </c>
+      <c r="G35" s="24" t="s">
+        <v>1078</v>
       </c>
     </row>
     <row r="36" spans="1:7">
       <c r="A36" t="s">
-        <v>993</v>
-      </c>
-      <c r="B36" s="49" t="s">
-        <v>1000</v>
-      </c>
-      <c r="C36" s="49" t="s">
-        <v>1001</v>
-      </c>
-      <c r="D36" s="49" t="s">
-        <v>428</v>
-      </c>
-      <c r="E36" s="46" t="s">
-        <v>1002</v>
-      </c>
-      <c r="F36" s="49" t="s">
-        <v>1003</v>
-      </c>
-      <c r="G36" s="46"/>
+        <v>1050</v>
+      </c>
+      <c r="B36" s="24" t="s">
+        <v>1079</v>
+      </c>
+      <c r="C36" s="24" t="s">
+        <v>1080</v>
+      </c>
+      <c r="D36" s="24" t="s">
+        <v>1081</v>
+      </c>
+      <c r="E36" s="109" t="s">
+        <v>1082</v>
+      </c>
+      <c r="F36" s="24" t="s">
+        <v>1083</v>
+      </c>
+      <c r="G36" s="24" t="s">
+        <v>1084</v>
+      </c>
     </row>
     <row r="37" spans="1:7">
       <c r="A37" t="s">
-        <v>993</v>
-      </c>
-      <c r="B37" s="49" t="s">
-        <v>1004</v>
-      </c>
-      <c r="C37" s="49" t="s">
-        <v>1005</v>
-      </c>
-      <c r="D37" s="49" t="s">
+        <v>1050</v>
+      </c>
+      <c r="B37" s="24" t="s">
+        <v>1085</v>
+      </c>
+      <c r="C37" s="24" t="s">
+        <v>1086</v>
+      </c>
+      <c r="D37" s="24" t="s">
         <v>428</v>
       </c>
-      <c r="E37" s="46" t="s">
-        <v>1006</v>
-      </c>
-      <c r="F37" s="49" t="s">
-        <v>1003</v>
-      </c>
-      <c r="G37" s="49" t="s">
-        <v>1007</v>
+      <c r="E37" s="109" t="s">
+        <v>1087</v>
+      </c>
+      <c r="F37" s="85" t="s">
+        <v>1088</v>
+      </c>
+      <c r="G37" s="109" t="s">
+        <v>1093</v>
       </c>
     </row>
     <row r="38" spans="1:7">
@@ -15713,319 +15719,199 @@
         <v>1050</v>
       </c>
       <c r="B38" s="24" t="s">
-        <v>1065</v>
+        <v>1089</v>
       </c>
       <c r="C38" s="24" t="s">
-        <v>1066</v>
+        <v>1090</v>
       </c>
       <c r="D38" s="24" t="s">
         <v>428</v>
       </c>
-      <c r="E38" s="109" t="s">
-        <v>1067</v>
+      <c r="E38" s="110" t="s">
+        <v>1091</v>
       </c>
       <c r="F38" s="24" t="s">
-        <v>1068</v>
-      </c>
-      <c r="G38" s="24" t="s">
-        <v>1069</v>
+        <v>1092</v>
+      </c>
+      <c r="G38" s="109" t="s">
+        <v>1094</v>
       </c>
     </row>
     <row r="39" spans="1:7">
       <c r="A39" t="s">
-        <v>1050</v>
-      </c>
-      <c r="B39" s="24" t="s">
-        <v>1070</v>
-      </c>
-      <c r="C39" s="24" t="s">
-        <v>1071</v>
-      </c>
-      <c r="D39" s="24" t="s">
+        <v>1183</v>
+      </c>
+      <c r="B39" s="49" t="s">
+        <v>1184</v>
+      </c>
+      <c r="C39" s="49" t="s">
+        <v>1185</v>
+      </c>
+      <c r="D39" s="49" t="s">
         <v>428</v>
       </c>
-      <c r="E39" s="109" t="s">
-        <v>1072</v>
-      </c>
-      <c r="F39" s="24" t="s">
-        <v>1073</v>
-      </c>
-      <c r="G39" s="24" t="s">
-        <v>1074</v>
+      <c r="E39" s="120" t="s">
+        <v>1186</v>
+      </c>
+      <c r="F39" s="49" t="s">
+        <v>1187</v>
+      </c>
+      <c r="G39" s="121" t="s">
+        <v>1188</v>
       </c>
     </row>
     <row r="40" spans="1:7">
       <c r="A40" t="s">
-        <v>1050</v>
-      </c>
-      <c r="B40" s="24" t="s">
-        <v>1075</v>
-      </c>
-      <c r="C40" s="24" t="s">
-        <v>1076</v>
-      </c>
-      <c r="D40" s="24" t="s">
+        <v>1183</v>
+      </c>
+      <c r="B40" s="49" t="s">
+        <v>1189</v>
+      </c>
+      <c r="C40" s="49" t="s">
+        <v>1190</v>
+      </c>
+      <c r="D40" s="49" t="s">
         <v>996</v>
       </c>
-      <c r="E40" s="109" t="s">
-        <v>1077</v>
-      </c>
-      <c r="F40" s="24" t="s">
-        <v>1073</v>
-      </c>
-      <c r="G40" s="24" t="s">
-        <v>1078</v>
+      <c r="E40" s="122" t="s">
+        <v>1191</v>
+      </c>
+      <c r="F40" s="49" t="s">
+        <v>1192</v>
+      </c>
+      <c r="G40" s="123" t="s">
+        <v>1193</v>
       </c>
     </row>
     <row r="41" spans="1:7">
       <c r="A41" t="s">
-        <v>1050</v>
-      </c>
-      <c r="B41" s="24" t="s">
-        <v>1079</v>
-      </c>
-      <c r="C41" s="24" t="s">
-        <v>1080</v>
-      </c>
-      <c r="D41" s="24" t="s">
-        <v>1081</v>
-      </c>
-      <c r="E41" s="109" t="s">
-        <v>1082</v>
-      </c>
-      <c r="F41" s="24" t="s">
-        <v>1083</v>
-      </c>
-      <c r="G41" s="24" t="s">
-        <v>1084</v>
+        <v>1055</v>
+      </c>
+      <c r="B41" s="130" t="s">
+        <v>1277</v>
+      </c>
+      <c r="C41" s="130" t="s">
+        <v>1278</v>
+      </c>
+      <c r="D41" s="130" t="s">
+        <v>1279</v>
+      </c>
+      <c r="E41" s="131" t="s">
+        <v>1280</v>
+      </c>
+      <c r="F41" s="130" t="s">
+        <v>1281</v>
+      </c>
+      <c r="G41" s="131" t="s">
+        <v>1286</v>
       </c>
     </row>
     <row r="42" spans="1:7">
       <c r="A42" t="s">
-        <v>1050</v>
-      </c>
-      <c r="B42" s="24" t="s">
-        <v>1085</v>
-      </c>
-      <c r="C42" s="24" t="s">
-        <v>1086</v>
-      </c>
-      <c r="D42" s="24" t="s">
-        <v>428</v>
-      </c>
-      <c r="E42" s="109" t="s">
-        <v>1087</v>
-      </c>
-      <c r="F42" s="85" t="s">
-        <v>1088</v>
-      </c>
-      <c r="G42" s="109" t="s">
-        <v>1093</v>
-      </c>
+        <v>1055</v>
+      </c>
+      <c r="B42" s="130" t="s">
+        <v>1282</v>
+      </c>
+      <c r="C42" s="130" t="s">
+        <v>1283</v>
+      </c>
+      <c r="D42" s="130"/>
+      <c r="E42" s="131" t="s">
+        <v>1284</v>
+      </c>
+      <c r="F42" s="130" t="s">
+        <v>1285</v>
+      </c>
+      <c r="G42" s="130"/>
     </row>
     <row r="43" spans="1:7">
       <c r="A43" t="s">
-        <v>1050</v>
-      </c>
-      <c r="B43" s="24" t="s">
-        <v>1089</v>
-      </c>
-      <c r="C43" s="24" t="s">
-        <v>1090</v>
-      </c>
-      <c r="D43" s="24" t="s">
-        <v>428</v>
-      </c>
-      <c r="E43" s="110" t="s">
-        <v>1091</v>
-      </c>
-      <c r="F43" s="24" t="s">
-        <v>1092</v>
-      </c>
-      <c r="G43" s="109" t="s">
-        <v>1094</v>
-      </c>
+        <v>1059</v>
+      </c>
+      <c r="B43" s="49" t="s">
+        <v>1377</v>
+      </c>
+      <c r="C43" s="49" t="s">
+        <v>1378</v>
+      </c>
+      <c r="D43" s="49"/>
+      <c r="E43" s="46" t="s">
+        <v>1379</v>
+      </c>
+      <c r="F43" s="49" t="s">
+        <v>1469</v>
+      </c>
+      <c r="G43" s="46"/>
     </row>
     <row r="44" spans="1:7">
       <c r="A44" t="s">
-        <v>1183</v>
+        <v>1059</v>
       </c>
       <c r="B44" s="49" t="s">
-        <v>1184</v>
+        <v>1380</v>
       </c>
       <c r="C44" s="49" t="s">
-        <v>1185</v>
+        <v>1381</v>
       </c>
       <c r="D44" s="49" t="s">
-        <v>428</v>
-      </c>
-      <c r="E44" s="120" t="s">
-        <v>1186</v>
+        <v>1382</v>
+      </c>
+      <c r="E44" s="46" t="s">
+        <v>1383</v>
       </c>
       <c r="F44" s="49" t="s">
-        <v>1187</v>
-      </c>
-      <c r="G44" s="121" t="s">
-        <v>1188</v>
-      </c>
-    </row>
-    <row r="45" spans="1:7">
-      <c r="A45" t="s">
-        <v>1183</v>
-      </c>
-      <c r="B45" s="49" t="s">
-        <v>1189</v>
-      </c>
-      <c r="C45" s="49" t="s">
-        <v>1190</v>
-      </c>
-      <c r="D45" s="49" t="s">
-        <v>996</v>
-      </c>
-      <c r="E45" s="122" t="s">
-        <v>1191</v>
-      </c>
-      <c r="F45" s="49" t="s">
-        <v>1192</v>
-      </c>
-      <c r="G45" s="123" t="s">
-        <v>1193</v>
-      </c>
-    </row>
-    <row r="46" spans="1:7">
-      <c r="A46" t="s">
-        <v>1055</v>
-      </c>
-      <c r="B46" s="130" t="s">
-        <v>1277</v>
-      </c>
-      <c r="C46" s="130" t="s">
-        <v>1278</v>
-      </c>
-      <c r="D46" s="130" t="s">
-        <v>1279</v>
-      </c>
-      <c r="E46" s="46" t="s">
-        <v>1280</v>
-      </c>
-      <c r="F46" s="130" t="s">
-        <v>1281</v>
-      </c>
-      <c r="G46" s="46" t="s">
-        <v>1286</v>
-      </c>
-    </row>
-    <row r="47" spans="1:7">
-      <c r="A47" t="s">
-        <v>1055</v>
-      </c>
-      <c r="B47" s="130" t="s">
-        <v>1282</v>
-      </c>
-      <c r="C47" s="130" t="s">
-        <v>1283</v>
-      </c>
-      <c r="D47" s="130"/>
-      <c r="E47" s="46" t="s">
-        <v>1284</v>
-      </c>
-      <c r="F47" s="130" t="s">
-        <v>1285</v>
-      </c>
-      <c r="G47" s="130"/>
-    </row>
-    <row r="48" spans="1:7">
-      <c r="A48" t="s">
-        <v>1059</v>
-      </c>
-      <c r="B48" s="49" t="s">
-        <v>1377</v>
-      </c>
-      <c r="C48" s="49" t="s">
-        <v>1378</v>
-      </c>
-      <c r="D48" s="49"/>
-      <c r="E48" s="46" t="s">
-        <v>1379</v>
-      </c>
-      <c r="F48" s="49" t="s">
-        <v>1469</v>
-      </c>
-      <c r="G48" s="46"/>
-    </row>
-    <row r="49" spans="1:7">
-      <c r="A49" t="s">
-        <v>1059</v>
-      </c>
-      <c r="B49" s="49" t="s">
-        <v>1380</v>
-      </c>
-      <c r="C49" s="49" t="s">
-        <v>1381</v>
-      </c>
-      <c r="D49" s="49" t="s">
-        <v>1382</v>
-      </c>
-      <c r="E49" s="46" t="s">
-        <v>1383</v>
-      </c>
-      <c r="F49" s="49" t="s">
         <v>1384</v>
       </c>
-      <c r="G49" s="46" t="s">
+      <c r="G44" s="46" t="s">
         <v>1385</v>
       </c>
     </row>
   </sheetData>
   <hyperlinks>
-    <hyperlink ref="E9" r:id="rId1" xr:uid="{E3CFFE38-E6D6-714C-8CB2-6C7908765724}"/>
-    <hyperlink ref="E10" r:id="rId2" xr:uid="{F2E60514-AAF2-A440-AE6A-F3B7A800911F}"/>
-    <hyperlink ref="E8" r:id="rId3" xr:uid="{B079DF0E-018E-9341-8C9C-61E8233F15E0}"/>
-    <hyperlink ref="E11" r:id="rId4" xr:uid="{1AC7D81A-6207-0940-9797-1B54146D29C9}"/>
-    <hyperlink ref="G13" r:id="rId5" display="https://orcid.org/0000-0001-6769-1983" xr:uid="{C44E8F08-6368-D74F-B1B2-A27AC4441576}"/>
-    <hyperlink ref="G12" r:id="rId6" display="https://orcid.org/0000-0003-2477-6869" xr:uid="{0489100D-EEF4-B949-AEFF-A6A4DC402620}"/>
-    <hyperlink ref="E21" r:id="rId7" xr:uid="{5F4E651F-562B-E24E-9CD1-9B3C1936C245}"/>
-    <hyperlink ref="E23" r:id="rId8" xr:uid="{F1125717-1141-4D42-A3A9-699125D01684}"/>
-    <hyperlink ref="E22" r:id="rId9" xr:uid="{1F332E72-AFB1-6744-B32C-C21F6FEBAA6E}"/>
-    <hyperlink ref="G21" r:id="rId10" display="https://orcid.org/0000-0002-1381-253X" xr:uid="{8EAB4384-125C-1B4B-BE58-8509C671817B}"/>
-    <hyperlink ref="E24" r:id="rId11" xr:uid="{87A5E650-E56F-F44A-8B6D-3500B47533C8}"/>
-    <hyperlink ref="E25" r:id="rId12" xr:uid="{BD2ECD0E-F5A3-804E-99C9-70ABA0785192}"/>
-    <hyperlink ref="G24" r:id="rId13" display="https://orcid.org/0000-0003-0951-780X" xr:uid="{DDA7CB87-9DEF-444A-B5E5-4DA5387FEAE7}"/>
-    <hyperlink ref="G25" r:id="rId14" display="https://orcid.org/0009-0007-7565-9714" xr:uid="{C3278E97-D66C-C04F-A534-F2DCF73A26A5}"/>
-    <hyperlink ref="E27" r:id="rId15" xr:uid="{A72A8784-3E65-CD4A-9CEA-D6821E18F4F0}"/>
-    <hyperlink ref="G26" r:id="rId16" display="https://orcid.org/0000-0003-4348-3690" xr:uid="{E9AFF3C1-A433-7741-A54F-44C2C489E5C4}"/>
+    <hyperlink ref="E4" r:id="rId1" xr:uid="{E3CFFE38-E6D6-714C-8CB2-6C7908765724}"/>
+    <hyperlink ref="E5" r:id="rId2" xr:uid="{F2E60514-AAF2-A440-AE6A-F3B7A800911F}"/>
+    <hyperlink ref="E3" r:id="rId3" xr:uid="{B079DF0E-018E-9341-8C9C-61E8233F15E0}"/>
+    <hyperlink ref="E6" r:id="rId4" xr:uid="{1AC7D81A-6207-0940-9797-1B54146D29C9}"/>
+    <hyperlink ref="G8" r:id="rId5" display="https://orcid.org/0000-0001-6769-1983" xr:uid="{C44E8F08-6368-D74F-B1B2-A27AC4441576}"/>
+    <hyperlink ref="G7" r:id="rId6" display="https://orcid.org/0000-0003-2477-6869" xr:uid="{0489100D-EEF4-B949-AEFF-A6A4DC402620}"/>
+    <hyperlink ref="E16" r:id="rId7" xr:uid="{5F4E651F-562B-E24E-9CD1-9B3C1936C245}"/>
+    <hyperlink ref="E18" r:id="rId8" xr:uid="{F1125717-1141-4D42-A3A9-699125D01684}"/>
+    <hyperlink ref="E17" r:id="rId9" xr:uid="{1F332E72-AFB1-6744-B32C-C21F6FEBAA6E}"/>
+    <hyperlink ref="G16" r:id="rId10" display="https://orcid.org/0000-0002-1381-253X" xr:uid="{8EAB4384-125C-1B4B-BE58-8509C671817B}"/>
+    <hyperlink ref="E19" r:id="rId11" xr:uid="{87A5E650-E56F-F44A-8B6D-3500B47533C8}"/>
+    <hyperlink ref="E20" r:id="rId12" xr:uid="{BD2ECD0E-F5A3-804E-99C9-70ABA0785192}"/>
+    <hyperlink ref="G19" r:id="rId13" display="https://orcid.org/0000-0003-0951-780X" xr:uid="{DDA7CB87-9DEF-444A-B5E5-4DA5387FEAE7}"/>
+    <hyperlink ref="G20" r:id="rId14" display="https://orcid.org/0009-0007-7565-9714" xr:uid="{C3278E97-D66C-C04F-A534-F2DCF73A26A5}"/>
+    <hyperlink ref="E22" r:id="rId15" xr:uid="{A72A8784-3E65-CD4A-9CEA-D6821E18F4F0}"/>
+    <hyperlink ref="G21" r:id="rId16" display="https://orcid.org/0000-0003-4348-3690" xr:uid="{E9AFF3C1-A433-7741-A54F-44C2C489E5C4}"/>
     <hyperlink ref="E2" r:id="rId17" xr:uid="{632BF422-FA2D-144A-9443-DEA9263E44B9}"/>
-    <hyperlink ref="G28" r:id="rId18" display="https://orcid.org/0000-0002-8726-306X" xr:uid="{84D128EF-A321-C14C-9A6C-47FF211C7B25}"/>
-    <hyperlink ref="E29" r:id="rId19" xr:uid="{CAB810DD-1FD3-D84E-B12A-6B1D1E12C04D}"/>
-    <hyperlink ref="G29" r:id="rId20" display="http://orcid.org/0000-0003-3535-7635" xr:uid="{E4794437-B59F-DB4C-B151-F9DDAECC9286}"/>
-    <hyperlink ref="E30" r:id="rId21" xr:uid="{E1B39D4A-FBDF-AB42-AFEC-5C4DBDFAE8A7}"/>
-    <hyperlink ref="G30" r:id="rId22" display="https://orcid.org/0000-0001-7604-0189" xr:uid="{4339A64C-035B-6245-919A-A8374AC5693D}"/>
-    <hyperlink ref="G31" r:id="rId23" display="https://orcid.org/0000-0001-7055-4701" xr:uid="{767A7D54-6548-E84D-981B-2EBD5369EDFF}"/>
-    <hyperlink ref="E32" r:id="rId24" xr:uid="{5E51343F-FF89-F14E-9FE3-8814A36D3C70}"/>
-    <hyperlink ref="E34" r:id="rId25" xr:uid="{A027007D-B16C-2D4A-A8C6-EE858E3A1D33}"/>
-    <hyperlink ref="E33" r:id="rId26" xr:uid="{DC6269BB-3246-D949-BC02-C59C24825789}"/>
-    <hyperlink ref="E35" r:id="rId27" xr:uid="{F9219FC4-650D-A647-94A8-FBD0AA56CFB7}"/>
-    <hyperlink ref="E36" r:id="rId28" xr:uid="{53118788-31F1-0149-8A20-F71DC03A8C9E}"/>
-    <hyperlink ref="E37" r:id="rId29" xr:uid="{6674C05C-673B-944F-98AB-75A0E6DAD5D7}"/>
-    <hyperlink ref="E38" r:id="rId30" xr:uid="{1E6CE376-85BC-EA4A-910D-DE1116AE6626}"/>
-    <hyperlink ref="E39" r:id="rId31" xr:uid="{8EE7483F-11FE-1248-B139-1CACB6186AA8}"/>
-    <hyperlink ref="E40" r:id="rId32" xr:uid="{77795DE8-0FC2-7341-81B6-278D1A2C4C8C}"/>
-    <hyperlink ref="E41" r:id="rId33" display="mailto:manon.de.deyne@vub.be" xr:uid="{AA5027B5-300A-F74C-B55B-E65732A75CDC}"/>
-    <hyperlink ref="E42" r:id="rId34" xr:uid="{C7E7CDCA-035E-1E4D-8532-EBEF677A2F25}"/>
-    <hyperlink ref="G42" r:id="rId35" display="https://orcid.org/0000-0002-1370-2090" xr:uid="{03A1AF0E-1F44-4940-A09A-56AB0017FB99}"/>
-    <hyperlink ref="E43" r:id="rId36" xr:uid="{1B1D269B-6E40-9748-A5C1-2D0CBA515977}"/>
-    <hyperlink ref="G43" r:id="rId37" display="https://orcid.org/0000-0001-9521-8085" xr:uid="{E54A6775-6C19-3A4B-BB48-482DD27FEE2E}"/>
-    <hyperlink ref="E44" r:id="rId38" xr:uid="{10759E79-85C3-DE40-8D6A-6C833FE92CB4}"/>
-    <hyperlink ref="G46" r:id="rId39" display="https://orcid.org/0000-0002-4202-4655" xr:uid="{848147C0-A9CA-E642-883A-ABE0683BC099}"/>
-    <hyperlink ref="E46" r:id="rId40" xr:uid="{1F029844-97BD-AA4C-B9EC-4978EC0229B0}"/>
-    <hyperlink ref="E47" r:id="rId41" xr:uid="{48E273F6-ED98-9A4D-B926-3360708B7FC2}"/>
-    <hyperlink ref="E48" r:id="rId42" xr:uid="{AF1B887C-35B7-8E4D-91D8-29E3CA5ACE86}"/>
-    <hyperlink ref="E49" r:id="rId43" xr:uid="{D9F36DA3-D0B7-7E42-85A4-528353BCA0E2}"/>
-    <hyperlink ref="E7" r:id="rId44" xr:uid="{40ED56F6-B773-AE47-ADE5-D486624FA922}"/>
-    <hyperlink ref="E6" r:id="rId45" xr:uid="{BFBCA679-676B-2142-9CF7-90BEE47AEF3C}"/>
-    <hyperlink ref="E5" r:id="rId46" xr:uid="{E288DD64-BDB2-F34C-8BDF-186D74BFA64F}"/>
-    <hyperlink ref="E3" r:id="rId47" xr:uid="{2D45CCE2-CA40-9942-AE5E-A35107A86068}"/>
-    <hyperlink ref="E4" r:id="rId48" xr:uid="{0DE5FBF5-CA34-7D4F-8638-16D4532F099F}"/>
+    <hyperlink ref="G23" r:id="rId18" display="https://orcid.org/0000-0002-8726-306X" xr:uid="{84D128EF-A321-C14C-9A6C-47FF211C7B25}"/>
+    <hyperlink ref="E24" r:id="rId19" xr:uid="{CAB810DD-1FD3-D84E-B12A-6B1D1E12C04D}"/>
+    <hyperlink ref="G24" r:id="rId20" display="http://orcid.org/0000-0003-3535-7635" xr:uid="{E4794437-B59F-DB4C-B151-F9DDAECC9286}"/>
+    <hyperlink ref="E25" r:id="rId21" xr:uid="{E1B39D4A-FBDF-AB42-AFEC-5C4DBDFAE8A7}"/>
+    <hyperlink ref="G25" r:id="rId22" display="https://orcid.org/0000-0001-7604-0189" xr:uid="{4339A64C-035B-6245-919A-A8374AC5693D}"/>
+    <hyperlink ref="G26" r:id="rId23" display="https://orcid.org/0000-0001-7055-4701" xr:uid="{767A7D54-6548-E84D-981B-2EBD5369EDFF}"/>
+    <hyperlink ref="E27" r:id="rId24" xr:uid="{5E51343F-FF89-F14E-9FE3-8814A36D3C70}"/>
+    <hyperlink ref="E29" r:id="rId25" xr:uid="{A027007D-B16C-2D4A-A8C6-EE858E3A1D33}"/>
+    <hyperlink ref="E28" r:id="rId26" xr:uid="{DC6269BB-3246-D949-BC02-C59C24825789}"/>
+    <hyperlink ref="E30" r:id="rId27" xr:uid="{F9219FC4-650D-A647-94A8-FBD0AA56CFB7}"/>
+    <hyperlink ref="E31" r:id="rId28" xr:uid="{53118788-31F1-0149-8A20-F71DC03A8C9E}"/>
+    <hyperlink ref="E32" r:id="rId29" xr:uid="{6674C05C-673B-944F-98AB-75A0E6DAD5D7}"/>
+    <hyperlink ref="E33" r:id="rId30" xr:uid="{1E6CE376-85BC-EA4A-910D-DE1116AE6626}"/>
+    <hyperlink ref="E34" r:id="rId31" xr:uid="{8EE7483F-11FE-1248-B139-1CACB6186AA8}"/>
+    <hyperlink ref="E35" r:id="rId32" xr:uid="{77795DE8-0FC2-7341-81B6-278D1A2C4C8C}"/>
+    <hyperlink ref="E36" r:id="rId33" display="mailto:manon.de.deyne@vub.be" xr:uid="{AA5027B5-300A-F74C-B55B-E65732A75CDC}"/>
+    <hyperlink ref="E37" r:id="rId34" xr:uid="{C7E7CDCA-035E-1E4D-8532-EBEF677A2F25}"/>
+    <hyperlink ref="G37" r:id="rId35" display="https://orcid.org/0000-0002-1370-2090" xr:uid="{03A1AF0E-1F44-4940-A09A-56AB0017FB99}"/>
+    <hyperlink ref="E38" r:id="rId36" xr:uid="{1B1D269B-6E40-9748-A5C1-2D0CBA515977}"/>
+    <hyperlink ref="G38" r:id="rId37" display="https://orcid.org/0000-0001-9521-8085" xr:uid="{E54A6775-6C19-3A4B-BB48-482DD27FEE2E}"/>
+    <hyperlink ref="E39" r:id="rId38" xr:uid="{10759E79-85C3-DE40-8D6A-6C833FE92CB4}"/>
+    <hyperlink ref="G41" r:id="rId39" display="https://orcid.org/0000-0002-4202-4655" xr:uid="{848147C0-A9CA-E642-883A-ABE0683BC099}"/>
+    <hyperlink ref="E41" r:id="rId40" xr:uid="{1F029844-97BD-AA4C-B9EC-4978EC0229B0}"/>
+    <hyperlink ref="E42" r:id="rId41" xr:uid="{48E273F6-ED98-9A4D-B926-3360708B7FC2}"/>
+    <hyperlink ref="E43" r:id="rId42" xr:uid="{AF1B887C-35B7-8E4D-91D8-29E3CA5ACE86}"/>
+    <hyperlink ref="E44" r:id="rId43" xr:uid="{D9F36DA3-D0B7-7E42-85A4-528353BCA0E2}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.78740157499999996" bottom="0.78740157499999996" header="0.3" footer="0.3"/>
 </worksheet>
@@ -16473,7 +16359,7 @@
         <v>126</v>
       </c>
     </row>
-    <row r="11" spans="1:6" ht="102">
+    <row r="11" spans="1:6" ht="119">
       <c r="A11" t="s">
         <v>209</v>
       </c>
@@ -16794,7 +16680,9 @@
       <c r="E1" t="s">
         <v>1012</v>
       </c>
-      <c r="F1"/>
+      <c r="F1" s="108" t="s">
+        <v>1470</v>
+      </c>
     </row>
     <row r="2" spans="1:6" ht="68">
       <c r="A2" s="12" t="s">
@@ -17246,7 +17134,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F1870FBA-EDD6-F747-8146-AD8380227C7B}">
-  <dimension ref="A1:E27"/>
+  <dimension ref="A1:F27"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="11.5" defaultRowHeight="16"/>
   <cols>
     <col min="1" max="1" width="33.83203125" style="25" customWidth="1"/>
@@ -17255,7 +17143,7 @@
     <col min="5" max="5" width="45.6640625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5">
+    <row r="1" spans="1:6">
       <c r="A1" t="s">
         <v>1013</v>
       </c>
@@ -17271,8 +17159,11 @@
       <c r="E1" t="s">
         <v>1017</v>
       </c>
-    </row>
-    <row r="2" spans="1:5" s="34" customFormat="1" ht="102">
+      <c r="F1" s="108" t="s">
+        <v>1471</v>
+      </c>
+    </row>
+    <row r="2" spans="1:6" s="34" customFormat="1" ht="119">
       <c r="A2" s="23" t="s">
         <v>405</v>
       </c>
@@ -17289,7 +17180,7 @@
         <v>418</v>
       </c>
     </row>
-    <row r="3" spans="1:5" ht="85">
+    <row r="3" spans="1:6" ht="85">
       <c r="A3" s="23" t="s">
         <v>405</v>
       </c>
@@ -17306,7 +17197,7 @@
         <v>415</v>
       </c>
     </row>
-    <row r="4" spans="1:5" ht="119">
+    <row r="4" spans="1:6" ht="119">
       <c r="A4" s="23" t="s">
         <v>405</v>
       </c>
@@ -17323,7 +17214,7 @@
         <v>412</v>
       </c>
     </row>
-    <row r="5" spans="1:5" ht="119">
+    <row r="5" spans="1:6" ht="119">
       <c r="A5" s="23" t="s">
         <v>405</v>
       </c>
@@ -17340,7 +17231,7 @@
         <v>409</v>
       </c>
     </row>
-    <row r="6" spans="1:5" ht="136">
+    <row r="6" spans="1:6" ht="136">
       <c r="A6" s="23" t="s">
         <v>405</v>
       </c>
@@ -17357,7 +17248,7 @@
         <v>406</v>
       </c>
     </row>
-    <row r="7" spans="1:5" ht="68">
+    <row r="7" spans="1:6" ht="68">
       <c r="A7" s="23" t="s">
         <v>405</v>
       </c>
@@ -17374,7 +17265,7 @@
         <v>402</v>
       </c>
     </row>
-    <row r="8" spans="1:5" ht="78" customHeight="1">
+    <row r="8" spans="1:6" ht="78" customHeight="1">
       <c r="A8" s="23" t="s">
         <v>395</v>
       </c>
@@ -17391,7 +17282,7 @@
         <v>399</v>
       </c>
     </row>
-    <row r="9" spans="1:5" ht="85">
+    <row r="9" spans="1:6" ht="85">
       <c r="A9" s="23" t="s">
         <v>395</v>
       </c>
@@ -17408,7 +17299,7 @@
         <v>396</v>
       </c>
     </row>
-    <row r="10" spans="1:5" ht="51">
+    <row r="10" spans="1:6" ht="51">
       <c r="A10" s="23" t="s">
         <v>395</v>
       </c>
@@ -17425,7 +17316,7 @@
         <v>392</v>
       </c>
     </row>
-    <row r="11" spans="1:5" ht="68">
+    <row r="11" spans="1:6" ht="68">
       <c r="A11" s="23" t="s">
         <v>361</v>
       </c>
@@ -17442,7 +17333,7 @@
         <v>389</v>
       </c>
     </row>
-    <row r="12" spans="1:5" ht="102">
+    <row r="12" spans="1:6" ht="102">
       <c r="A12" s="23" t="s">
         <v>361</v>
       </c>
@@ -17459,7 +17350,7 @@
         <v>386</v>
       </c>
     </row>
-    <row r="13" spans="1:5" ht="68">
+    <row r="13" spans="1:6" ht="68">
       <c r="A13" s="23" t="s">
         <v>361</v>
       </c>
@@ -17476,7 +17367,7 @@
         <v>383</v>
       </c>
     </row>
-    <row r="14" spans="1:5" ht="51">
+    <row r="14" spans="1:6" ht="51">
       <c r="A14" s="23" t="s">
         <v>361</v>
       </c>
@@ -17493,7 +17384,7 @@
         <v>380</v>
       </c>
     </row>
-    <row r="15" spans="1:5" ht="85">
+    <row r="15" spans="1:6" ht="102">
       <c r="A15" s="23" t="s">
         <v>361</v>
       </c>
@@ -17510,7 +17401,7 @@
         <v>377</v>
       </c>
     </row>
-    <row r="16" spans="1:5" ht="51">
+    <row r="16" spans="1:6" ht="51">
       <c r="A16" s="23" t="s">
         <v>361</v>
       </c>
@@ -17721,7 +17612,7 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5E08B14F-287D-9E4F-82CD-595A79363C01}">
-  <dimension ref="A1:E27"/>
+  <dimension ref="A1:F27"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="11.5" defaultRowHeight="16"/>
   <cols>
     <col min="1" max="1" width="49.6640625" customWidth="1"/>
@@ -17729,7 +17620,7 @@
     <col min="3" max="5" width="42.33203125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5">
+    <row r="1" spans="1:6">
       <c r="A1" t="s">
         <v>1018</v>
       </c>
@@ -17745,8 +17636,11 @@
       <c r="E1" t="s">
         <v>1022</v>
       </c>
-    </row>
-    <row r="2" spans="1:5" s="34" customFormat="1" ht="119">
+      <c r="F1" s="108" t="s">
+        <v>1472</v>
+      </c>
+    </row>
+    <row r="2" spans="1:6" s="34" customFormat="1" ht="119">
       <c r="A2" s="41" t="s">
         <v>541</v>
       </c>
@@ -17763,7 +17657,7 @@
         <v>551</v>
       </c>
     </row>
-    <row r="3" spans="1:5" ht="170">
+    <row r="3" spans="1:6" ht="170">
       <c r="A3" s="41" t="s">
         <v>541</v>
       </c>
@@ -17780,7 +17674,7 @@
         <v>548</v>
       </c>
     </row>
-    <row r="4" spans="1:5" ht="221">
+    <row r="4" spans="1:6" ht="221">
       <c r="A4" s="41" t="s">
         <v>541</v>
       </c>
@@ -17797,7 +17691,7 @@
         <v>545</v>
       </c>
     </row>
-    <row r="5" spans="1:5" ht="102">
+    <row r="5" spans="1:6" ht="102">
       <c r="A5" s="41" t="s">
         <v>541</v>
       </c>
@@ -17814,7 +17708,7 @@
         <v>542</v>
       </c>
     </row>
-    <row r="6" spans="1:5" ht="153">
+    <row r="6" spans="1:6" ht="153">
       <c r="A6" s="41" t="s">
         <v>541</v>
       </c>
@@ -17831,7 +17725,7 @@
         <v>538</v>
       </c>
     </row>
-    <row r="7" spans="1:5" ht="102">
+    <row r="7" spans="1:6" ht="102">
       <c r="A7" s="41" t="s">
         <v>537</v>
       </c>
@@ -17848,7 +17742,7 @@
         <v>534</v>
       </c>
     </row>
-    <row r="8" spans="1:5" ht="119">
+    <row r="8" spans="1:6" ht="119">
       <c r="A8" s="41" t="s">
         <v>527</v>
       </c>
@@ -17865,7 +17759,7 @@
         <v>531</v>
       </c>
     </row>
-    <row r="9" spans="1:5" ht="102">
+    <row r="9" spans="1:6" ht="119">
       <c r="A9" s="41" t="s">
         <v>527</v>
       </c>
@@ -17882,7 +17776,7 @@
         <v>528</v>
       </c>
     </row>
-    <row r="10" spans="1:5" ht="85">
+    <row r="10" spans="1:6" ht="85">
       <c r="A10" s="41" t="s">
         <v>527</v>
       </c>
@@ -17899,7 +17793,7 @@
         <v>524</v>
       </c>
     </row>
-    <row r="11" spans="1:5" ht="68">
+    <row r="11" spans="1:6" ht="68">
       <c r="A11" s="41" t="s">
         <v>493</v>
       </c>
@@ -17916,7 +17810,7 @@
         <v>521</v>
       </c>
     </row>
-    <row r="12" spans="1:5" ht="102">
+    <row r="12" spans="1:6" ht="102">
       <c r="A12" s="41" t="s">
         <v>493</v>
       </c>
@@ -17933,7 +17827,7 @@
         <v>518</v>
       </c>
     </row>
-    <row r="13" spans="1:5" ht="68">
+    <row r="13" spans="1:6" ht="68">
       <c r="A13" s="41" t="s">
         <v>493</v>
       </c>
@@ -17950,7 +17844,7 @@
         <v>515</v>
       </c>
     </row>
-    <row r="14" spans="1:5" ht="68">
+    <row r="14" spans="1:6" ht="68">
       <c r="A14" s="41" t="s">
         <v>493</v>
       </c>
@@ -17967,7 +17861,7 @@
         <v>512</v>
       </c>
     </row>
-    <row r="15" spans="1:5" ht="102">
+    <row r="15" spans="1:6" ht="102">
       <c r="A15" s="41" t="s">
         <v>493</v>
       </c>
@@ -17984,7 +17878,7 @@
         <v>509</v>
       </c>
     </row>
-    <row r="16" spans="1:5" ht="68">
+    <row r="16" spans="1:6" ht="68">
       <c r="A16" s="41" t="s">
         <v>493</v>
       </c>
@@ -18195,7 +18089,7 @@
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{DD1BAFA5-BB3F-3746-96CA-1E15CD5F496C}">
-  <dimension ref="A1:E27"/>
+  <dimension ref="A1:F27"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="13.33203125" defaultRowHeight="18"/>
   <cols>
     <col min="1" max="1" width="58" style="53" customWidth="1"/>
@@ -18204,7 +18098,7 @@
     <col min="6" max="16384" width="13.33203125" style="52"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5">
+    <row r="1" spans="1:6">
       <c r="A1" t="s">
         <v>1033</v>
       </c>
@@ -18220,8 +18114,11 @@
       <c r="E1" t="s">
         <v>1037</v>
       </c>
-    </row>
-    <row r="2" spans="1:5" ht="76">
+      <c r="F1" s="108" t="s">
+        <v>1473</v>
+      </c>
+    </row>
+    <row r="2" spans="1:6" ht="76">
       <c r="A2" s="57" t="s">
         <v>661</v>
       </c>
@@ -18238,7 +18135,7 @@
         <v>674</v>
       </c>
     </row>
-    <row r="3" spans="1:5" ht="57">
+    <row r="3" spans="1:6" ht="57">
       <c r="A3" s="57" t="s">
         <v>661</v>
       </c>
@@ -18255,7 +18152,7 @@
         <v>671</v>
       </c>
     </row>
-    <row r="4" spans="1:5" ht="114">
+    <row r="4" spans="1:6" ht="114">
       <c r="A4" s="57" t="s">
         <v>661</v>
       </c>
@@ -18272,7 +18169,7 @@
         <v>668</v>
       </c>
     </row>
-    <row r="5" spans="1:5" ht="76">
+    <row r="5" spans="1:6" ht="76">
       <c r="A5" s="57" t="s">
         <v>661</v>
       </c>
@@ -18289,7 +18186,7 @@
         <v>665</v>
       </c>
     </row>
-    <row r="6" spans="1:5" ht="76">
+    <row r="6" spans="1:6" ht="76">
       <c r="A6" s="57" t="s">
         <v>661</v>
       </c>
@@ -18306,7 +18203,7 @@
         <v>662</v>
       </c>
     </row>
-    <row r="7" spans="1:5" ht="58.5" customHeight="1">
+    <row r="7" spans="1:6" ht="58.5" customHeight="1">
       <c r="A7" s="57" t="s">
         <v>661</v>
       </c>
@@ -18323,7 +18220,7 @@
         <v>658</v>
       </c>
     </row>
-    <row r="8" spans="1:5" ht="57">
+    <row r="8" spans="1:6" ht="57">
       <c r="A8" s="57" t="s">
         <v>651</v>
       </c>
@@ -18340,7 +18237,7 @@
         <v>655</v>
       </c>
     </row>
-    <row r="9" spans="1:5" ht="76">
+    <row r="9" spans="1:6" ht="76">
       <c r="A9" s="57" t="s">
         <v>651</v>
       </c>
@@ -18357,7 +18254,7 @@
         <v>652</v>
       </c>
     </row>
-    <row r="10" spans="1:5" ht="38">
+    <row r="10" spans="1:6" ht="38">
       <c r="A10" s="57" t="s">
         <v>651</v>
       </c>
@@ -18374,7 +18271,7 @@
         <v>648</v>
       </c>
     </row>
-    <row r="11" spans="1:5" ht="38">
+    <row r="11" spans="1:6" ht="38">
       <c r="A11" s="57" t="s">
         <v>617</v>
       </c>
@@ -18391,7 +18288,7 @@
         <v>645</v>
       </c>
     </row>
-    <row r="12" spans="1:5" ht="76">
+    <row r="12" spans="1:6" ht="76">
       <c r="A12" s="57" t="s">
         <v>617</v>
       </c>
@@ -18408,7 +18305,7 @@
         <v>642</v>
       </c>
     </row>
-    <row r="13" spans="1:5" ht="57">
+    <row r="13" spans="1:6" ht="57">
       <c r="A13" s="57" t="s">
         <v>617</v>
       </c>
@@ -18425,7 +18322,7 @@
         <v>639</v>
       </c>
     </row>
-    <row r="14" spans="1:5" ht="57">
+    <row r="14" spans="1:6" ht="57">
       <c r="A14" s="57" t="s">
         <v>617</v>
       </c>
@@ -18442,7 +18339,7 @@
         <v>636</v>
       </c>
     </row>
-    <row r="15" spans="1:5" ht="57">
+    <row r="15" spans="1:6" ht="57">
       <c r="A15" s="57" t="s">
         <v>617</v>
       </c>
@@ -18459,7 +18356,7 @@
         <v>633</v>
       </c>
     </row>
-    <row r="16" spans="1:5" ht="57">
+    <row r="16" spans="1:6" ht="57">
       <c r="A16" s="57" t="s">
         <v>617</v>
       </c>
@@ -18646,7 +18543,7 @@
         <v>598</v>
       </c>
     </row>
-    <row r="27" spans="1:5" ht="77" thickBot="1">
+    <row r="27" spans="1:5" ht="96" thickBot="1">
       <c r="A27" s="57" t="s">
         <v>597</v>
       </c>
@@ -18696,6 +18593,9 @@
       <c r="E1" t="s">
         <v>1027</v>
       </c>
+      <c r="F1" s="108" t="s">
+        <v>1474</v>
+      </c>
     </row>
     <row r="2" spans="1:22" ht="102">
       <c r="A2" s="72" t="s">
@@ -19164,7 +19064,7 @@
 
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1A873EFD-FDC9-F34B-9E47-4FB43415AA3A}">
-  <dimension ref="A1:E27"/>
+  <dimension ref="A1:F27"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="11.5" defaultRowHeight="16"/>
   <cols>
     <col min="1" max="1" width="49.6640625" customWidth="1"/>
@@ -19172,7 +19072,7 @@
     <col min="3" max="5" width="42.33203125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5">
+    <row r="1" spans="1:6">
       <c r="A1" t="s">
         <v>1038</v>
       </c>
@@ -19188,8 +19088,11 @@
       <c r="E1" t="s">
         <v>1042</v>
       </c>
-    </row>
-    <row r="2" spans="1:5" s="34" customFormat="1" ht="102">
+      <c r="F1" s="108" t="s">
+        <v>1475</v>
+      </c>
+    </row>
+    <row r="2" spans="1:6" s="34" customFormat="1" ht="102">
       <c r="A2" s="23" t="s">
         <v>904</v>
       </c>
@@ -19206,7 +19109,7 @@
         <v>901</v>
       </c>
     </row>
-    <row r="3" spans="1:5" ht="85">
+    <row r="3" spans="1:6" ht="85">
       <c r="A3" s="23" t="s">
         <v>904</v>
       </c>
@@ -19223,7 +19126,7 @@
         <v>898</v>
       </c>
     </row>
-    <row r="4" spans="1:5" ht="119">
+    <row r="4" spans="1:6" ht="119">
       <c r="A4" s="23" t="s">
         <v>904</v>
       </c>
@@ -19240,7 +19143,7 @@
         <v>895</v>
       </c>
     </row>
-    <row r="5" spans="1:5" ht="136">
+    <row r="5" spans="1:6" ht="136">
       <c r="A5" s="23" t="s">
         <v>904</v>
       </c>
@@ -19257,7 +19160,7 @@
         <v>892</v>
       </c>
     </row>
-    <row r="6" spans="1:5" ht="136">
+    <row r="6" spans="1:6" ht="136">
       <c r="A6" s="23" t="s">
         <v>904</v>
       </c>
@@ -19274,7 +19177,7 @@
         <v>889</v>
       </c>
     </row>
-    <row r="7" spans="1:5" ht="95">
+    <row r="7" spans="1:6" ht="95">
       <c r="A7" s="23" t="s">
         <v>904</v>
       </c>
@@ -19291,7 +19194,7 @@
         <v>886</v>
       </c>
     </row>
-    <row r="8" spans="1:5" ht="102">
+    <row r="8" spans="1:6" ht="102">
       <c r="A8" s="23" t="s">
         <v>885</v>
       </c>
@@ -19308,7 +19211,7 @@
         <v>882</v>
       </c>
     </row>
-    <row r="9" spans="1:5" ht="85">
+    <row r="9" spans="1:6" ht="85">
       <c r="A9" s="23" t="s">
         <v>885</v>
       </c>
@@ -19325,7 +19228,7 @@
         <v>879</v>
       </c>
     </row>
-    <row r="10" spans="1:5" ht="57">
+    <row r="10" spans="1:6" ht="57">
       <c r="A10" s="23" t="s">
         <v>885</v>
       </c>
@@ -19342,7 +19245,7 @@
         <v>876</v>
       </c>
     </row>
-    <row r="11" spans="1:5" ht="85">
+    <row r="11" spans="1:6" ht="85">
       <c r="A11" s="23" t="s">
         <v>875</v>
       </c>
@@ -19359,7 +19262,7 @@
         <v>872</v>
       </c>
     </row>
-    <row r="12" spans="1:5" ht="119">
+    <row r="12" spans="1:6" ht="119">
       <c r="A12" s="23" t="s">
         <v>875</v>
       </c>
@@ -19376,7 +19279,7 @@
         <v>869</v>
       </c>
     </row>
-    <row r="13" spans="1:5" ht="76">
+    <row r="13" spans="1:6" ht="76">
       <c r="A13" s="23" t="s">
         <v>875</v>
       </c>
@@ -19393,7 +19296,7 @@
         <v>866</v>
       </c>
     </row>
-    <row r="14" spans="1:5" ht="76">
+    <row r="14" spans="1:6" ht="76">
       <c r="A14" s="23" t="s">
         <v>875</v>
       </c>
@@ -19410,7 +19313,7 @@
         <v>863</v>
       </c>
     </row>
-    <row r="15" spans="1:5" ht="85">
+    <row r="15" spans="1:6" ht="102">
       <c r="A15" s="23" t="s">
         <v>875</v>
       </c>
@@ -19427,7 +19330,7 @@
         <v>860</v>
       </c>
     </row>
-    <row r="16" spans="1:5" ht="68">
+    <row r="16" spans="1:6" ht="68">
       <c r="A16" s="23" t="s">
         <v>875</v>
       </c>
@@ -19495,7 +19398,7 @@
         <v>848</v>
       </c>
     </row>
-    <row r="20" spans="1:5" ht="68">
+    <row r="20" spans="1:5" ht="85">
       <c r="A20" s="23" t="s">
         <v>875</v>
       </c>
@@ -19512,7 +19415,7 @@
         <v>845</v>
       </c>
     </row>
-    <row r="21" spans="1:5" ht="95">
+    <row r="21" spans="1:5" ht="114">
       <c r="A21" s="23" t="s">
         <v>875</v>
       </c>
@@ -19597,7 +19500,7 @@
         <v>828</v>
       </c>
     </row>
-    <row r="26" spans="1:5" ht="119">
+    <row r="26" spans="1:5" ht="136">
       <c r="A26" s="23" t="s">
         <v>831</v>
       </c>
@@ -19638,7 +19541,7 @@
 
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{73049A3F-8369-7B4D-8239-B0CE97E178CB}">
-  <dimension ref="A1:E27"/>
+  <dimension ref="A1:F27"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="11.5" defaultRowHeight="16"/>
   <cols>
     <col min="1" max="1" width="28.5" customWidth="1"/>
@@ -19646,7 +19549,7 @@
     <col min="3" max="5" width="42.33203125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5">
+    <row r="1" spans="1:6">
       <c r="A1" t="s">
         <v>1028</v>
       </c>
@@ -19662,8 +19565,11 @@
       <c r="E1" t="s">
         <v>1032</v>
       </c>
-    </row>
-    <row r="2" spans="1:5" s="34" customFormat="1" ht="51">
+      <c r="F1" s="108" t="s">
+        <v>1476</v>
+      </c>
+    </row>
+    <row r="2" spans="1:6" s="34" customFormat="1" ht="51">
       <c r="A2" s="23" t="s">
         <v>972</v>
       </c>
@@ -19680,7 +19586,7 @@
         <v>985</v>
       </c>
     </row>
-    <row r="3" spans="1:5" ht="68">
+    <row r="3" spans="1:6" ht="68">
       <c r="A3" s="23" t="s">
         <v>972</v>
       </c>
@@ -19697,7 +19603,7 @@
         <v>982</v>
       </c>
     </row>
-    <row r="4" spans="1:5" ht="68">
+    <row r="4" spans="1:6" ht="68">
       <c r="A4" s="23" t="s">
         <v>972</v>
       </c>
@@ -19714,7 +19620,7 @@
         <v>979</v>
       </c>
     </row>
-    <row r="5" spans="1:5" ht="85">
+    <row r="5" spans="1:6" ht="85">
       <c r="A5" s="23" t="s">
         <v>972</v>
       </c>
@@ -19731,7 +19637,7 @@
         <v>976</v>
       </c>
     </row>
-    <row r="6" spans="1:5" ht="68">
+    <row r="6" spans="1:6" ht="68">
       <c r="A6" s="23" t="s">
         <v>972</v>
       </c>
@@ -19748,7 +19654,7 @@
         <v>973</v>
       </c>
     </row>
-    <row r="7" spans="1:5" ht="34">
+    <row r="7" spans="1:6" ht="34">
       <c r="A7" s="23" t="s">
         <v>972</v>
       </c>
@@ -19765,7 +19671,7 @@
         <v>969</v>
       </c>
     </row>
-    <row r="8" spans="1:5" ht="68">
+    <row r="8" spans="1:6" ht="68">
       <c r="A8" s="23" t="s">
         <v>962</v>
       </c>
@@ -19782,7 +19688,7 @@
         <v>966</v>
       </c>
     </row>
-    <row r="9" spans="1:5" ht="68">
+    <row r="9" spans="1:6" ht="68">
       <c r="A9" s="23" t="s">
         <v>962</v>
       </c>
@@ -19799,7 +19705,7 @@
         <v>963</v>
       </c>
     </row>
-    <row r="10" spans="1:5" ht="34">
+    <row r="10" spans="1:6" ht="34">
       <c r="A10" s="23" t="s">
         <v>962</v>
       </c>
@@ -19816,7 +19722,7 @@
         <v>959</v>
       </c>
     </row>
-    <row r="11" spans="1:5" ht="51">
+    <row r="11" spans="1:6" ht="51">
       <c r="A11" s="23" t="s">
         <v>928</v>
       </c>
@@ -19833,7 +19739,7 @@
         <v>956</v>
       </c>
     </row>
-    <row r="12" spans="1:5" ht="85">
+    <row r="12" spans="1:6" ht="85">
       <c r="A12" s="23" t="s">
         <v>928</v>
       </c>
@@ -19850,7 +19756,7 @@
         <v>953</v>
       </c>
     </row>
-    <row r="13" spans="1:5" ht="34">
+    <row r="13" spans="1:6" ht="34">
       <c r="A13" s="23" t="s">
         <v>928</v>
       </c>
@@ -19867,7 +19773,7 @@
         <v>950</v>
       </c>
     </row>
-    <row r="14" spans="1:5" ht="34">
+    <row r="14" spans="1:6" ht="34">
       <c r="A14" s="23" t="s">
         <v>928</v>
       </c>
@@ -19884,7 +19790,7 @@
         <v>947</v>
       </c>
     </row>
-    <row r="15" spans="1:5" ht="68">
+    <row r="15" spans="1:6" ht="68">
       <c r="A15" s="23" t="s">
         <v>928</v>
       </c>
@@ -19901,7 +19807,7 @@
         <v>944</v>
       </c>
     </row>
-    <row r="16" spans="1:5" ht="34">
+    <row r="16" spans="1:6" ht="34">
       <c r="A16" s="23" t="s">
         <v>928</v>
       </c>

</xml_diff>